<commit_message>
[Feat] Lingjack Migration Script
</commit_message>
<xml_diff>
--- a/SWO/Raw Script/swo.xlsx
+++ b/SWO/Raw Script/swo.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="11003"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jordan/Alitec/docker/odoo18/repo/lingjack-import-script/SWO/Raw Script/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACD914B0-9C6F-7C4E-A93E-A5CB3F4C523E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="795" windowWidth="29040" windowHeight="16440"/>
+    <workbookView xWindow="0" yWindow="800" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Outstanding SWO Listing" sheetId="1" r:id="rId1"/>
@@ -976,7 +982,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1476,7 +1482,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1495,10 +1501,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1558,9 +1560,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1598,7 +1600,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -1670,7 +1672,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1843,29 +1845,29 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Q406"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="7.140625" customWidth="1"/>
-    <col min="2" max="2" width="25.42578125" style="3" customWidth="1"/>
-    <col min="3" max="3" width="18.28515625" customWidth="1"/>
-    <col min="4" max="4" width="11.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="33.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="30.140625" style="7" customWidth="1"/>
-    <col min="7" max="7" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.85546875" customWidth="1"/>
-    <col min="9" max="9" width="30.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="36.42578125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="22.7109375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="26.28515625" style="3" customWidth="1"/>
+    <col min="1" max="1" width="7.1640625" customWidth="1"/>
+    <col min="2" max="2" width="25.5" style="3" customWidth="1"/>
+    <col min="3" max="3" width="18.33203125" customWidth="1"/>
+    <col min="4" max="4" width="11.5" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="33.5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="30.1640625" style="7" customWidth="1"/>
+    <col min="7" max="7" width="16.5" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.83203125" customWidth="1"/>
+    <col min="9" max="9" width="30.5" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.1640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="36.5" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="22.6640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="26.33203125" style="3" customWidth="1"/>
     <col min="14" max="14" width="24" style="3" customWidth="1"/>
-    <col min="15" max="15" width="18.7109375" style="9" bestFit="1" customWidth="1"/>
-    <col min="16" max="17" width="28.85546875" customWidth="1"/>
+    <col min="15" max="15" width="18.6640625" bestFit="1" customWidth="1"/>
+    <col min="16" max="17" width="28.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1908,7 +1910,7 @@
       <c r="N1" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="O1" s="8" t="s">
+      <c r="O1" s="1" t="s">
         <v>11</v>
       </c>
       <c r="P1" s="1" t="s">
@@ -1918,7 +1920,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:17" ht="51.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" ht="45" x14ac:dyDescent="0.2">
       <c r="A2" s="2"/>
       <c r="B2" s="5" t="s">
         <v>21</v>
@@ -1966,7 +1968,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="3" spans="1:17" ht="51.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:17" ht="60" x14ac:dyDescent="0.2">
       <c r="A3" s="2"/>
       <c r="B3" s="5" t="s">
         <v>26</v>
@@ -2014,7 +2016,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="4" spans="1:17" ht="77.25" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:17" ht="75" x14ac:dyDescent="0.2">
       <c r="A4" s="2"/>
       <c r="B4" s="5" t="s">
         <v>34</v>
@@ -2062,7 +2064,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="5" spans="1:17" ht="39" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:17" ht="45" x14ac:dyDescent="0.2">
       <c r="A5" s="2"/>
       <c r="B5" s="5" t="s">
         <v>253</v>
@@ -2108,7 +2110,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="6" spans="1:17" ht="51.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:17" ht="45" x14ac:dyDescent="0.2">
       <c r="A6" s="2"/>
       <c r="B6" s="5" t="s">
         <v>18</v>
@@ -2151,7 +2153,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="7" spans="1:17" ht="64.5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:17" ht="60" x14ac:dyDescent="0.2">
       <c r="A7" s="2"/>
       <c r="B7" s="5" t="s">
         <v>23</v>
@@ -2199,7 +2201,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="8" spans="1:17" ht="51.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:17" ht="60" x14ac:dyDescent="0.2">
       <c r="A8" s="2"/>
       <c r="B8" s="5" t="s">
         <v>29</v>
@@ -2244,7 +2246,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="9" spans="1:17" ht="51.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:17" ht="45" x14ac:dyDescent="0.2">
       <c r="A9" s="2"/>
       <c r="B9" s="5" t="s">
         <v>253</v>
@@ -2290,7 +2292,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="10" spans="1:17" ht="26.25" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A10" s="2"/>
       <c r="B10" s="5" t="s">
         <v>16</v>
@@ -2336,7 +2338,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="11" spans="1:17" ht="26.25" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A11" s="2"/>
       <c r="B11" s="5" t="s">
         <v>16</v>
@@ -2382,7 +2384,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="12" spans="1:17" ht="51.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:17" ht="60" x14ac:dyDescent="0.2">
       <c r="A12" s="2"/>
       <c r="B12" s="5" t="s">
         <v>20</v>
@@ -2430,7 +2432,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="13" spans="1:17" ht="64.5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:17" ht="60" x14ac:dyDescent="0.2">
       <c r="A13" s="2"/>
       <c r="B13" s="5" t="s">
         <v>32</v>
@@ -2478,7 +2480,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="14" spans="1:17" ht="64.5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:17" ht="60" x14ac:dyDescent="0.2">
       <c r="A14" s="2"/>
       <c r="B14" s="5" t="s">
         <v>31</v>
@@ -2526,7 +2528,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="15" spans="1:17" ht="51.75" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:17" ht="45" x14ac:dyDescent="0.2">
       <c r="A15" s="2"/>
       <c r="B15" s="5" t="s">
         <v>19</v>
@@ -2574,7 +2576,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="16" spans="1:17" ht="64.5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:17" ht="60" x14ac:dyDescent="0.2">
       <c r="A16" s="2"/>
       <c r="B16" s="5" t="s">
         <v>32</v>
@@ -2622,7 +2624,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="17" spans="1:16" ht="64.5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:16" ht="60" x14ac:dyDescent="0.2">
       <c r="A17" s="2"/>
       <c r="B17" s="5" t="s">
         <v>254</v>
@@ -2670,7 +2672,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="18" spans="1:16" ht="39" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:16" ht="45" x14ac:dyDescent="0.2">
       <c r="A18" s="2"/>
       <c r="B18" s="5" t="s">
         <v>16</v>
@@ -2716,7 +2718,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="19" spans="1:16" ht="64.5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:16" ht="60" x14ac:dyDescent="0.2">
       <c r="A19" s="2"/>
       <c r="B19" s="5" t="s">
         <v>23</v>
@@ -2764,7 +2766,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="20" spans="1:16" ht="64.5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:16" ht="75" x14ac:dyDescent="0.2">
       <c r="A20" s="2"/>
       <c r="B20" s="5" t="s">
         <v>34</v>
@@ -2812,7 +2814,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="21" spans="1:16" ht="51.75" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:16" ht="45" x14ac:dyDescent="0.2">
       <c r="A21" s="2"/>
       <c r="B21" s="5" t="s">
         <v>15</v>
@@ -2860,7 +2862,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="22" spans="1:16" ht="90" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:16" ht="90" x14ac:dyDescent="0.2">
       <c r="A22" s="2"/>
       <c r="B22" s="5" t="s">
         <v>34</v>
@@ -2908,7 +2910,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="23" spans="1:16" ht="51.75" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:16" ht="60" x14ac:dyDescent="0.2">
       <c r="A23" s="2"/>
       <c r="B23" s="5" t="s">
         <v>27</v>
@@ -2953,7 +2955,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="24" spans="1:16" ht="51.75" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:16" ht="45" x14ac:dyDescent="0.2">
       <c r="A24" s="2"/>
       <c r="B24" s="5" t="s">
         <v>255</v>
@@ -3001,7 +3003,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="25" spans="1:16" ht="51.75" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:16" ht="60" x14ac:dyDescent="0.2">
       <c r="A25" s="2"/>
       <c r="B25" s="5" t="s">
         <v>25</v>
@@ -3049,7 +3051,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="26" spans="1:16" ht="51.75" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:16" ht="60" x14ac:dyDescent="0.2">
       <c r="A26" s="2"/>
       <c r="B26" s="5" t="s">
         <v>34</v>
@@ -3097,7 +3099,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="27" spans="1:16" ht="77.25" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:16" ht="75" x14ac:dyDescent="0.2">
       <c r="A27" s="2"/>
       <c r="B27" s="5" t="s">
         <v>33</v>
@@ -3142,7 +3144,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="28" spans="1:16" ht="102.75" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:16" ht="105" x14ac:dyDescent="0.2">
       <c r="A28" s="2"/>
       <c r="B28" s="5" t="s">
         <v>34</v>
@@ -3190,7 +3192,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="29" spans="1:16" ht="64.5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:16" ht="60" x14ac:dyDescent="0.2">
       <c r="A29" s="2"/>
       <c r="B29" s="5" t="s">
         <v>30</v>
@@ -3235,7 +3237,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="30" spans="1:16" ht="64.5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:16" ht="60" x14ac:dyDescent="0.2">
       <c r="A30" s="2"/>
       <c r="B30" s="5" t="s">
         <v>32</v>
@@ -3283,7 +3285,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="31" spans="1:16" ht="77.25" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:16" ht="75" x14ac:dyDescent="0.2">
       <c r="A31" s="2"/>
       <c r="B31" s="5" t="s">
         <v>34</v>
@@ -3331,7 +3333,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="32" spans="1:16" ht="26.25" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A32" s="2"/>
       <c r="B32" s="5" t="s">
         <v>35</v>
@@ -3377,7 +3379,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="33" spans="1:17" ht="39" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:17" ht="30" x14ac:dyDescent="0.2">
       <c r="A33" s="2"/>
       <c r="B33" s="5" t="s">
         <v>256</v>
@@ -3422,7 +3424,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="34" spans="1:17" ht="64.5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:17" ht="60" x14ac:dyDescent="0.2">
       <c r="A34" s="2"/>
       <c r="B34" s="5" t="s">
         <v>28</v>
@@ -3473,7 +3475,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="35" spans="1:17" ht="64.5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:17" ht="60" x14ac:dyDescent="0.2">
       <c r="A35" s="2"/>
       <c r="B35" s="5" t="s">
         <v>257</v>
@@ -3518,7 +3520,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="36" spans="1:17" ht="26.25" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A36" s="2"/>
       <c r="B36" s="5" t="s">
         <v>35</v>
@@ -3564,7 +3566,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="37" spans="1:17" ht="51.75" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:17" ht="60" x14ac:dyDescent="0.2">
       <c r="A37" s="2"/>
       <c r="B37" s="5" t="s">
         <v>258</v>
@@ -3609,7 +3611,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="38" spans="1:17" ht="64.5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:17" ht="60" x14ac:dyDescent="0.2">
       <c r="A38" s="2"/>
       <c r="B38" s="5" t="s">
         <v>259</v>
@@ -3657,7 +3659,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="39" spans="1:17" ht="64.5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:17" ht="60" x14ac:dyDescent="0.2">
       <c r="A39" s="2"/>
       <c r="B39" s="5" t="s">
         <v>36</v>
@@ -3702,7 +3704,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="40" spans="1:17" ht="77.25" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:17" ht="75" x14ac:dyDescent="0.2">
       <c r="A40" s="2"/>
       <c r="B40" s="5" t="s">
         <v>260</v>
@@ -3747,7 +3749,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="41" spans="1:17" ht="51.75" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:17" ht="45" x14ac:dyDescent="0.2">
       <c r="A41" s="2"/>
       <c r="B41" s="5" t="s">
         <v>261</v>
@@ -3795,7 +3797,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="42" spans="1:17" ht="51.75" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:17" ht="60" x14ac:dyDescent="0.2">
       <c r="A42" s="2"/>
       <c r="B42" s="5" t="s">
         <v>24</v>
@@ -3843,7 +3845,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="43" spans="1:17" ht="51.75" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:17" ht="45" x14ac:dyDescent="0.2">
       <c r="A43" s="2"/>
       <c r="B43" s="5" t="s">
         <v>17</v>
@@ -3891,7 +3893,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="44" spans="1:17" ht="77.25" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:17" ht="75" x14ac:dyDescent="0.2">
       <c r="A44" s="2"/>
       <c r="B44" s="5" t="s">
         <v>22</v>
@@ -3936,7 +3938,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="45" spans="1:17" ht="26.25" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A45" s="2"/>
       <c r="B45" s="5" t="s">
         <v>262</v>
@@ -3981,7 +3983,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="46" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A46" s="2"/>
       <c r="B46" s="5"/>
       <c r="C46" s="2"/>
@@ -3997,7 +3999,7 @@
       <c r="N46" s="5"/>
       <c r="O46" s="2"/>
     </row>
-    <row r="47" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A47" s="2"/>
       <c r="B47" s="5"/>
       <c r="C47" s="2"/>
@@ -4013,7 +4015,7 @@
       <c r="N47" s="5"/>
       <c r="O47" s="2"/>
     </row>
-    <row r="48" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A48" s="2"/>
       <c r="B48" s="5"/>
       <c r="C48" s="2"/>
@@ -4029,7 +4031,7 @@
       <c r="N48" s="5"/>
       <c r="O48" s="2"/>
     </row>
-    <row r="49" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A49" s="2"/>
       <c r="B49" s="5"/>
       <c r="C49" s="2"/>
@@ -4045,7 +4047,7 @@
       <c r="N49" s="5"/>
       <c r="O49" s="2"/>
     </row>
-    <row r="50" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A50" s="2"/>
       <c r="B50" s="5"/>
       <c r="C50" s="2"/>
@@ -4061,7 +4063,7 @@
       <c r="N50" s="5"/>
       <c r="O50" s="2"/>
     </row>
-    <row r="51" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A51" s="2"/>
       <c r="B51" s="5"/>
       <c r="C51" s="2"/>
@@ -4077,7 +4079,7 @@
       <c r="N51" s="5"/>
       <c r="O51" s="2"/>
     </row>
-    <row r="52" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A52" s="2"/>
       <c r="B52" s="5"/>
       <c r="C52" s="2"/>
@@ -4093,7 +4095,7 @@
       <c r="N52" s="5"/>
       <c r="O52" s="2"/>
     </row>
-    <row r="53" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A53" s="2"/>
       <c r="B53" s="5"/>
       <c r="C53" s="2"/>
@@ -4109,7 +4111,7 @@
       <c r="N53" s="5"/>
       <c r="O53" s="2"/>
     </row>
-    <row r="54" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A54" s="2"/>
       <c r="B54" s="5"/>
       <c r="C54" s="2"/>
@@ -4125,7 +4127,7 @@
       <c r="N54" s="5"/>
       <c r="O54" s="2"/>
     </row>
-    <row r="55" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A55" s="2"/>
       <c r="B55" s="5"/>
       <c r="C55" s="2"/>
@@ -4141,7 +4143,7 @@
       <c r="N55" s="5"/>
       <c r="O55" s="2"/>
     </row>
-    <row r="56" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A56" s="2"/>
       <c r="B56" s="5"/>
       <c r="C56" s="2"/>
@@ -4157,7 +4159,7 @@
       <c r="N56" s="5"/>
       <c r="O56" s="2"/>
     </row>
-    <row r="57" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A57" s="2"/>
       <c r="B57" s="5"/>
       <c r="C57" s="2"/>
@@ -4173,7 +4175,7 @@
       <c r="N57" s="5"/>
       <c r="O57" s="2"/>
     </row>
-    <row r="58" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A58" s="2"/>
       <c r="B58" s="5"/>
       <c r="C58" s="2"/>
@@ -4189,7 +4191,7 @@
       <c r="N58" s="5"/>
       <c r="O58" s="2"/>
     </row>
-    <row r="59" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A59" s="2"/>
       <c r="B59" s="5"/>
       <c r="C59" s="2"/>
@@ -4205,7 +4207,7 @@
       <c r="N59" s="5"/>
       <c r="O59" s="2"/>
     </row>
-    <row r="60" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A60" s="2"/>
       <c r="B60" s="5"/>
       <c r="C60" s="2"/>
@@ -4221,7 +4223,7 @@
       <c r="N60" s="5"/>
       <c r="O60" s="2"/>
     </row>
-    <row r="61" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A61" s="2"/>
       <c r="B61" s="5"/>
       <c r="C61" s="2"/>
@@ -4237,7 +4239,7 @@
       <c r="N61" s="5"/>
       <c r="O61" s="2"/>
     </row>
-    <row r="62" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A62" s="2"/>
       <c r="B62" s="5"/>
       <c r="C62" s="2"/>
@@ -4253,7 +4255,7 @@
       <c r="N62" s="5"/>
       <c r="O62" s="2"/>
     </row>
-    <row r="63" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A63" s="2"/>
       <c r="B63" s="5"/>
       <c r="C63" s="2"/>
@@ -4269,7 +4271,7 @@
       <c r="N63" s="5"/>
       <c r="O63" s="2"/>
     </row>
-    <row r="64" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A64" s="2"/>
       <c r="B64" s="5"/>
       <c r="C64" s="2"/>
@@ -4285,7 +4287,7 @@
       <c r="N64" s="5"/>
       <c r="O64" s="2"/>
     </row>
-    <row r="65" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A65" s="2"/>
       <c r="B65" s="5"/>
       <c r="C65" s="2"/>
@@ -4301,7 +4303,7 @@
       <c r="N65" s="5"/>
       <c r="O65" s="2"/>
     </row>
-    <row r="66" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A66" s="2"/>
       <c r="B66" s="5"/>
       <c r="C66" s="2"/>
@@ -4317,7 +4319,7 @@
       <c r="N66" s="5"/>
       <c r="O66" s="2"/>
     </row>
-    <row r="67" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A67" s="2"/>
       <c r="B67" s="5"/>
       <c r="C67" s="2"/>
@@ -4333,7 +4335,7 @@
       <c r="N67" s="5"/>
       <c r="O67" s="2"/>
     </row>
-    <row r="68" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A68" s="2"/>
       <c r="B68" s="5"/>
       <c r="C68" s="2"/>
@@ -4349,7 +4351,7 @@
       <c r="N68" s="5"/>
       <c r="O68" s="2"/>
     </row>
-    <row r="69" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A69" s="2"/>
       <c r="B69" s="5"/>
       <c r="C69" s="2"/>
@@ -4365,7 +4367,7 @@
       <c r="N69" s="5"/>
       <c r="O69" s="2"/>
     </row>
-    <row r="70" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A70" s="2"/>
       <c r="B70" s="5"/>
       <c r="C70" s="2"/>
@@ -4381,7 +4383,7 @@
       <c r="N70" s="5"/>
       <c r="O70" s="2"/>
     </row>
-    <row r="71" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A71" s="2"/>
       <c r="B71" s="5"/>
       <c r="C71" s="2"/>
@@ -4397,7 +4399,7 @@
       <c r="N71" s="5"/>
       <c r="O71" s="2"/>
     </row>
-    <row r="72" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A72" s="2"/>
       <c r="B72" s="5"/>
       <c r="C72" s="2"/>
@@ -4413,7 +4415,7 @@
       <c r="N72" s="5"/>
       <c r="O72" s="2"/>
     </row>
-    <row r="73" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A73" s="2"/>
       <c r="B73" s="5"/>
       <c r="C73" s="2"/>
@@ -4429,7 +4431,7 @@
       <c r="N73" s="5"/>
       <c r="O73" s="2"/>
     </row>
-    <row r="74" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A74" s="2"/>
       <c r="B74" s="5"/>
       <c r="C74" s="2"/>
@@ -4445,7 +4447,7 @@
       <c r="N74" s="5"/>
       <c r="O74" s="2"/>
     </row>
-    <row r="75" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A75" s="2"/>
       <c r="B75" s="5"/>
       <c r="C75" s="2"/>
@@ -4461,7 +4463,7 @@
       <c r="N75" s="5"/>
       <c r="O75" s="2"/>
     </row>
-    <row r="76" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A76" s="2"/>
       <c r="B76" s="5"/>
       <c r="C76" s="2"/>
@@ -4477,7 +4479,7 @@
       <c r="N76" s="5"/>
       <c r="O76" s="2"/>
     </row>
-    <row r="77" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A77" s="2"/>
       <c r="B77" s="5"/>
       <c r="C77" s="2"/>
@@ -4493,7 +4495,7 @@
       <c r="N77" s="5"/>
       <c r="O77" s="2"/>
     </row>
-    <row r="78" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A78" s="2"/>
       <c r="B78" s="5"/>
       <c r="C78" s="2"/>
@@ -4509,7 +4511,7 @@
       <c r="N78" s="5"/>
       <c r="O78" s="2"/>
     </row>
-    <row r="79" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A79" s="2"/>
       <c r="B79" s="5"/>
       <c r="C79" s="2"/>
@@ -4525,7 +4527,7 @@
       <c r="N79" s="5"/>
       <c r="O79" s="2"/>
     </row>
-    <row r="80" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A80" s="2"/>
       <c r="B80" s="5"/>
       <c r="C80" s="2"/>
@@ -4541,7 +4543,7 @@
       <c r="N80" s="5"/>
       <c r="O80" s="2"/>
     </row>
-    <row r="81" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A81" s="2"/>
       <c r="B81" s="5"/>
       <c r="C81" s="2"/>
@@ -4557,7 +4559,7 @@
       <c r="N81" s="5"/>
       <c r="O81" s="2"/>
     </row>
-    <row r="82" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A82" s="2"/>
       <c r="B82" s="5"/>
       <c r="C82" s="2"/>
@@ -4573,7 +4575,7 @@
       <c r="N82" s="5"/>
       <c r="O82" s="2"/>
     </row>
-    <row r="83" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A83" s="2"/>
       <c r="B83" s="5"/>
       <c r="C83" s="2"/>
@@ -4589,7 +4591,7 @@
       <c r="N83" s="5"/>
       <c r="O83" s="2"/>
     </row>
-    <row r="84" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A84" s="2"/>
       <c r="B84" s="5"/>
       <c r="C84" s="2"/>
@@ -4605,7 +4607,7 @@
       <c r="N84" s="5"/>
       <c r="O84" s="2"/>
     </row>
-    <row r="85" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A85" s="2"/>
       <c r="B85" s="5"/>
       <c r="C85" s="2"/>
@@ -4621,7 +4623,7 @@
       <c r="N85" s="5"/>
       <c r="O85" s="2"/>
     </row>
-    <row r="86" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A86" s="2"/>
       <c r="B86" s="5"/>
       <c r="C86" s="2"/>
@@ -4637,7 +4639,7 @@
       <c r="N86" s="5"/>
       <c r="O86" s="2"/>
     </row>
-    <row r="87" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A87" s="2"/>
       <c r="B87" s="5"/>
       <c r="C87" s="2"/>
@@ -4653,7 +4655,7 @@
       <c r="N87" s="5"/>
       <c r="O87" s="2"/>
     </row>
-    <row r="88" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A88" s="2"/>
       <c r="B88" s="5"/>
       <c r="C88" s="2"/>
@@ -4669,7 +4671,7 @@
       <c r="N88" s="5"/>
       <c r="O88" s="2"/>
     </row>
-    <row r="89" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A89" s="2"/>
       <c r="B89" s="5"/>
       <c r="C89" s="2"/>
@@ -4685,7 +4687,7 @@
       <c r="N89" s="5"/>
       <c r="O89" s="2"/>
     </row>
-    <row r="90" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A90" s="2"/>
       <c r="B90" s="5"/>
       <c r="C90" s="2"/>
@@ -4701,7 +4703,7 @@
       <c r="N90" s="5"/>
       <c r="O90" s="2"/>
     </row>
-    <row r="91" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A91" s="2"/>
       <c r="B91" s="5"/>
       <c r="C91" s="2"/>
@@ -4717,7 +4719,7 @@
       <c r="N91" s="5"/>
       <c r="O91" s="2"/>
     </row>
-    <row r="92" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A92" s="2"/>
       <c r="B92" s="5"/>
       <c r="C92" s="2"/>
@@ -4733,7 +4735,7 @@
       <c r="N92" s="5"/>
       <c r="O92" s="2"/>
     </row>
-    <row r="93" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A93" s="2"/>
       <c r="B93" s="5"/>
       <c r="C93" s="2"/>
@@ -4749,7 +4751,7 @@
       <c r="N93" s="5"/>
       <c r="O93" s="2"/>
     </row>
-    <row r="94" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A94" s="2"/>
       <c r="B94" s="5"/>
       <c r="C94" s="2"/>
@@ -4765,7 +4767,7 @@
       <c r="N94" s="5"/>
       <c r="O94" s="2"/>
     </row>
-    <row r="95" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A95" s="2"/>
       <c r="B95" s="5"/>
       <c r="C95" s="2"/>
@@ -4781,7 +4783,7 @@
       <c r="N95" s="5"/>
       <c r="O95" s="2"/>
     </row>
-    <row r="96" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A96" s="2"/>
       <c r="B96" s="5"/>
       <c r="C96" s="2"/>
@@ -4797,7 +4799,7 @@
       <c r="N96" s="5"/>
       <c r="O96" s="2"/>
     </row>
-    <row r="97" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A97" s="2"/>
       <c r="B97" s="5"/>
       <c r="C97" s="2"/>
@@ -4813,7 +4815,7 @@
       <c r="N97" s="5"/>
       <c r="O97" s="2"/>
     </row>
-    <row r="98" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A98" s="2"/>
       <c r="B98" s="5"/>
       <c r="C98" s="2"/>
@@ -4829,7 +4831,7 @@
       <c r="N98" s="5"/>
       <c r="O98" s="2"/>
     </row>
-    <row r="99" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A99" s="2"/>
       <c r="B99" s="5"/>
       <c r="C99" s="2"/>
@@ -4845,7 +4847,7 @@
       <c r="N99" s="5"/>
       <c r="O99" s="2"/>
     </row>
-    <row r="100" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A100" s="2"/>
       <c r="B100" s="5"/>
       <c r="C100" s="2"/>
@@ -4861,7 +4863,7 @@
       <c r="N100" s="5"/>
       <c r="O100" s="2"/>
     </row>
-    <row r="101" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A101" s="2"/>
       <c r="B101" s="5"/>
       <c r="C101" s="2"/>
@@ -4877,7 +4879,7 @@
       <c r="N101" s="5"/>
       <c r="O101" s="2"/>
     </row>
-    <row r="102" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A102" s="2"/>
       <c r="B102" s="5"/>
       <c r="C102" s="2"/>
@@ -4893,7 +4895,7 @@
       <c r="N102" s="5"/>
       <c r="O102" s="2"/>
     </row>
-    <row r="103" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A103" s="2"/>
       <c r="B103" s="5"/>
       <c r="C103" s="2"/>
@@ -4909,7 +4911,7 @@
       <c r="N103" s="5"/>
       <c r="O103" s="2"/>
     </row>
-    <row r="104" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A104" s="2"/>
       <c r="B104" s="5"/>
       <c r="C104" s="2"/>
@@ -4925,7 +4927,7 @@
       <c r="N104" s="5"/>
       <c r="O104" s="2"/>
     </row>
-    <row r="105" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A105" s="2"/>
       <c r="B105" s="5"/>
       <c r="C105" s="2"/>
@@ -4941,7 +4943,7 @@
       <c r="N105" s="5"/>
       <c r="O105" s="2"/>
     </row>
-    <row r="106" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A106" s="2"/>
       <c r="B106" s="5"/>
       <c r="C106" s="2"/>
@@ -4957,7 +4959,7 @@
       <c r="N106" s="5"/>
       <c r="O106" s="2"/>
     </row>
-    <row r="107" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A107" s="2"/>
       <c r="B107" s="5"/>
       <c r="C107" s="2"/>
@@ -4973,7 +4975,7 @@
       <c r="N107" s="5"/>
       <c r="O107" s="2"/>
     </row>
-    <row r="108" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A108" s="2"/>
       <c r="B108" s="5"/>
       <c r="C108" s="2"/>
@@ -4989,7 +4991,7 @@
       <c r="N108" s="5"/>
       <c r="O108" s="2"/>
     </row>
-    <row r="109" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A109" s="2"/>
       <c r="B109" s="5"/>
       <c r="C109" s="2"/>
@@ -5005,7 +5007,7 @@
       <c r="N109" s="5"/>
       <c r="O109" s="2"/>
     </row>
-    <row r="110" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A110" s="2"/>
       <c r="B110" s="5"/>
       <c r="C110" s="2"/>
@@ -5021,7 +5023,7 @@
       <c r="N110" s="5"/>
       <c r="O110" s="2"/>
     </row>
-    <row r="111" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A111" s="2"/>
       <c r="B111" s="5"/>
       <c r="C111" s="2"/>
@@ -5037,7 +5039,7 @@
       <c r="N111" s="5"/>
       <c r="O111" s="2"/>
     </row>
-    <row r="112" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A112" s="2"/>
       <c r="B112" s="5"/>
       <c r="C112" s="2"/>
@@ -5053,7 +5055,7 @@
       <c r="N112" s="5"/>
       <c r="O112" s="2"/>
     </row>
-    <row r="113" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A113" s="2"/>
       <c r="B113" s="5"/>
       <c r="C113" s="2"/>
@@ -5069,7 +5071,7 @@
       <c r="N113" s="5"/>
       <c r="O113" s="2"/>
     </row>
-    <row r="114" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A114" s="2"/>
       <c r="B114" s="5"/>
       <c r="C114" s="2"/>
@@ -5085,7 +5087,7 @@
       <c r="N114" s="5"/>
       <c r="O114" s="2"/>
     </row>
-    <row r="115" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A115" s="2"/>
       <c r="B115" s="5"/>
       <c r="C115" s="2"/>
@@ -5101,7 +5103,7 @@
       <c r="N115" s="5"/>
       <c r="O115" s="2"/>
     </row>
-    <row r="116" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A116" s="2"/>
       <c r="B116" s="5"/>
       <c r="C116" s="2"/>
@@ -5117,7 +5119,7 @@
       <c r="N116" s="5"/>
       <c r="O116" s="2"/>
     </row>
-    <row r="117" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A117" s="2"/>
       <c r="B117" s="5"/>
       <c r="C117" s="2"/>
@@ -5133,7 +5135,7 @@
       <c r="N117" s="5"/>
       <c r="O117" s="2"/>
     </row>
-    <row r="118" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A118" s="2"/>
       <c r="B118" s="5"/>
       <c r="C118" s="2"/>
@@ -5149,7 +5151,7 @@
       <c r="N118" s="5"/>
       <c r="O118" s="2"/>
     </row>
-    <row r="119" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A119" s="2"/>
       <c r="B119" s="5"/>
       <c r="C119" s="2"/>
@@ -5165,7 +5167,7 @@
       <c r="N119" s="5"/>
       <c r="O119" s="2"/>
     </row>
-    <row r="120" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A120" s="2"/>
       <c r="B120" s="5"/>
       <c r="C120" s="2"/>
@@ -5181,7 +5183,7 @@
       <c r="N120" s="5"/>
       <c r="O120" s="2"/>
     </row>
-    <row r="121" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A121" s="2"/>
       <c r="B121" s="5"/>
       <c r="C121" s="2"/>
@@ -5197,7 +5199,7 @@
       <c r="N121" s="5"/>
       <c r="O121" s="2"/>
     </row>
-    <row r="122" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A122" s="2"/>
       <c r="B122" s="5"/>
       <c r="C122" s="2"/>
@@ -5213,7 +5215,7 @@
       <c r="N122" s="5"/>
       <c r="O122" s="2"/>
     </row>
-    <row r="123" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A123" s="2"/>
       <c r="B123" s="5"/>
       <c r="C123" s="2"/>
@@ -5229,7 +5231,7 @@
       <c r="N123" s="5"/>
       <c r="O123" s="2"/>
     </row>
-    <row r="124" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A124" s="2"/>
       <c r="B124" s="5"/>
       <c r="C124" s="2"/>
@@ -5245,7 +5247,7 @@
       <c r="N124" s="5"/>
       <c r="O124" s="2"/>
     </row>
-    <row r="125" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A125" s="2"/>
       <c r="B125" s="5"/>
       <c r="C125" s="2"/>
@@ -5261,7 +5263,7 @@
       <c r="N125" s="5"/>
       <c r="O125" s="2"/>
     </row>
-    <row r="126" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A126" s="2"/>
       <c r="B126" s="5"/>
       <c r="C126" s="2"/>
@@ -5277,7 +5279,7 @@
       <c r="N126" s="5"/>
       <c r="O126" s="2"/>
     </row>
-    <row r="127" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A127" s="2"/>
       <c r="B127" s="5"/>
       <c r="C127" s="2"/>
@@ -5293,7 +5295,7 @@
       <c r="N127" s="5"/>
       <c r="O127" s="2"/>
     </row>
-    <row r="128" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A128" s="2"/>
       <c r="B128" s="5"/>
       <c r="C128" s="2"/>
@@ -5309,7 +5311,7 @@
       <c r="N128" s="5"/>
       <c r="O128" s="2"/>
     </row>
-    <row r="129" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A129" s="2"/>
       <c r="B129" s="5"/>
       <c r="C129" s="2"/>
@@ -5325,7 +5327,7 @@
       <c r="N129" s="5"/>
       <c r="O129" s="2"/>
     </row>
-    <row r="130" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A130" s="2"/>
       <c r="B130" s="5"/>
       <c r="C130" s="2"/>
@@ -5341,7 +5343,7 @@
       <c r="N130" s="5"/>
       <c r="O130" s="2"/>
     </row>
-    <row r="131" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A131" s="2"/>
       <c r="B131" s="5"/>
       <c r="C131" s="2"/>
@@ -5357,7 +5359,7 @@
       <c r="N131" s="5"/>
       <c r="O131" s="2"/>
     </row>
-    <row r="132" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A132" s="2"/>
       <c r="B132" s="5"/>
       <c r="C132" s="2"/>
@@ -5373,7 +5375,7 @@
       <c r="N132" s="5"/>
       <c r="O132" s="2"/>
     </row>
-    <row r="133" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A133" s="2"/>
       <c r="B133" s="5"/>
       <c r="C133" s="2"/>
@@ -5389,7 +5391,7 @@
       <c r="N133" s="5"/>
       <c r="O133" s="2"/>
     </row>
-    <row r="134" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A134" s="2"/>
       <c r="B134" s="5"/>
       <c r="C134" s="2"/>
@@ -5405,7 +5407,7 @@
       <c r="N134" s="5"/>
       <c r="O134" s="2"/>
     </row>
-    <row r="135" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A135" s="2"/>
       <c r="B135" s="5"/>
       <c r="C135" s="2"/>
@@ -5421,7 +5423,7 @@
       <c r="N135" s="5"/>
       <c r="O135" s="2"/>
     </row>
-    <row r="136" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A136" s="2"/>
       <c r="B136" s="5"/>
       <c r="C136" s="2"/>
@@ -5437,7 +5439,7 @@
       <c r="N136" s="5"/>
       <c r="O136" s="2"/>
     </row>
-    <row r="137" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A137" s="2"/>
       <c r="B137" s="5"/>
       <c r="C137" s="2"/>
@@ -5453,7 +5455,7 @@
       <c r="N137" s="5"/>
       <c r="O137" s="2"/>
     </row>
-    <row r="138" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A138" s="2"/>
       <c r="B138" s="5"/>
       <c r="C138" s="2"/>
@@ -5469,7 +5471,7 @@
       <c r="N138" s="5"/>
       <c r="O138" s="2"/>
     </row>
-    <row r="139" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A139" s="2"/>
       <c r="B139" s="5"/>
       <c r="C139" s="2"/>
@@ -5485,7 +5487,7 @@
       <c r="N139" s="5"/>
       <c r="O139" s="2"/>
     </row>
-    <row r="140" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A140" s="2"/>
       <c r="B140" s="5"/>
       <c r="C140" s="2"/>
@@ -5501,7 +5503,7 @@
       <c r="N140" s="5"/>
       <c r="O140" s="2"/>
     </row>
-    <row r="141" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A141" s="2"/>
       <c r="B141" s="5"/>
       <c r="C141" s="2"/>
@@ -5517,7 +5519,7 @@
       <c r="N141" s="5"/>
       <c r="O141" s="2"/>
     </row>
-    <row r="142" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A142" s="2"/>
       <c r="B142" s="5"/>
       <c r="C142" s="2"/>
@@ -5533,7 +5535,7 @@
       <c r="N142" s="5"/>
       <c r="O142" s="2"/>
     </row>
-    <row r="143" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A143" s="2"/>
       <c r="B143" s="5"/>
       <c r="C143" s="2"/>
@@ -5549,7 +5551,7 @@
       <c r="N143" s="5"/>
       <c r="O143" s="2"/>
     </row>
-    <row r="144" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A144" s="2"/>
       <c r="B144" s="5"/>
       <c r="C144" s="2"/>
@@ -5565,7 +5567,7 @@
       <c r="N144" s="5"/>
       <c r="O144" s="2"/>
     </row>
-    <row r="145" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A145" s="2"/>
       <c r="B145" s="5"/>
       <c r="C145" s="2"/>
@@ -5581,7 +5583,7 @@
       <c r="N145" s="5"/>
       <c r="O145" s="2"/>
     </row>
-    <row r="146" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A146" s="2"/>
       <c r="B146" s="5"/>
       <c r="C146" s="2"/>
@@ -5597,7 +5599,7 @@
       <c r="N146" s="5"/>
       <c r="O146" s="2"/>
     </row>
-    <row r="147" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A147" s="2"/>
       <c r="B147" s="5"/>
       <c r="C147" s="2"/>
@@ -5613,7 +5615,7 @@
       <c r="N147" s="5"/>
       <c r="O147" s="2"/>
     </row>
-    <row r="148" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A148" s="2"/>
       <c r="B148" s="5"/>
       <c r="C148" s="2"/>
@@ -5629,7 +5631,7 @@
       <c r="N148" s="5"/>
       <c r="O148" s="2"/>
     </row>
-    <row r="149" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A149" s="2"/>
       <c r="B149" s="5"/>
       <c r="C149" s="2"/>
@@ -5645,7 +5647,7 @@
       <c r="N149" s="5"/>
       <c r="O149" s="2"/>
     </row>
-    <row r="150" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A150" s="2"/>
       <c r="B150" s="5"/>
       <c r="C150" s="2"/>
@@ -5661,7 +5663,7 @@
       <c r="N150" s="5"/>
       <c r="O150" s="2"/>
     </row>
-    <row r="151" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A151" s="2"/>
       <c r="B151" s="5"/>
       <c r="C151" s="2"/>
@@ -5677,7 +5679,7 @@
       <c r="N151" s="5"/>
       <c r="O151" s="2"/>
     </row>
-    <row r="152" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A152" s="2"/>
       <c r="B152" s="5"/>
       <c r="C152" s="2"/>
@@ -5693,7 +5695,7 @@
       <c r="N152" s="5"/>
       <c r="O152" s="2"/>
     </row>
-    <row r="153" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A153" s="2"/>
       <c r="B153" s="5"/>
       <c r="C153" s="2"/>
@@ -5709,7 +5711,7 @@
       <c r="N153" s="5"/>
       <c r="O153" s="2"/>
     </row>
-    <row r="154" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A154" s="2"/>
       <c r="B154" s="5"/>
       <c r="C154" s="2"/>
@@ -5725,7 +5727,7 @@
       <c r="N154" s="5"/>
       <c r="O154" s="2"/>
     </row>
-    <row r="155" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A155" s="2"/>
       <c r="B155" s="5"/>
       <c r="C155" s="2"/>
@@ -5741,7 +5743,7 @@
       <c r="N155" s="5"/>
       <c r="O155" s="2"/>
     </row>
-    <row r="156" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A156" s="2"/>
       <c r="B156" s="5"/>
       <c r="C156" s="2"/>
@@ -5757,7 +5759,7 @@
       <c r="N156" s="5"/>
       <c r="O156" s="2"/>
     </row>
-    <row r="157" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A157" s="2"/>
       <c r="B157" s="5"/>
       <c r="C157" s="2"/>
@@ -5773,7 +5775,7 @@
       <c r="N157" s="5"/>
       <c r="O157" s="2"/>
     </row>
-    <row r="158" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A158" s="2"/>
       <c r="B158" s="5"/>
       <c r="C158" s="2"/>
@@ -5789,7 +5791,7 @@
       <c r="N158" s="5"/>
       <c r="O158" s="2"/>
     </row>
-    <row r="159" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A159" s="2"/>
       <c r="B159" s="5"/>
       <c r="C159" s="2"/>
@@ -5805,7 +5807,7 @@
       <c r="N159" s="5"/>
       <c r="O159" s="2"/>
     </row>
-    <row r="160" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A160" s="2"/>
       <c r="B160" s="5"/>
       <c r="C160" s="2"/>
@@ -5821,7 +5823,7 @@
       <c r="N160" s="5"/>
       <c r="O160" s="2"/>
     </row>
-    <row r="161" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A161" s="2"/>
       <c r="B161" s="5"/>
       <c r="C161" s="2"/>
@@ -5837,7 +5839,7 @@
       <c r="N161" s="5"/>
       <c r="O161" s="2"/>
     </row>
-    <row r="162" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A162" s="2"/>
       <c r="B162" s="5"/>
       <c r="C162" s="2"/>
@@ -5853,7 +5855,7 @@
       <c r="N162" s="5"/>
       <c r="O162" s="2"/>
     </row>
-    <row r="163" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A163" s="2"/>
       <c r="B163" s="5"/>
       <c r="C163" s="2"/>
@@ -5869,7 +5871,7 @@
       <c r="N163" s="5"/>
       <c r="O163" s="2"/>
     </row>
-    <row r="164" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A164" s="2"/>
       <c r="B164" s="5"/>
       <c r="C164" s="2"/>
@@ -5885,7 +5887,7 @@
       <c r="N164" s="5"/>
       <c r="O164" s="2"/>
     </row>
-    <row r="165" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A165" s="2"/>
       <c r="B165" s="5"/>
       <c r="C165" s="2"/>
@@ -5901,7 +5903,7 @@
       <c r="N165" s="5"/>
       <c r="O165" s="2"/>
     </row>
-    <row r="166" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A166" s="2"/>
       <c r="B166" s="5"/>
       <c r="C166" s="2"/>
@@ -5917,7 +5919,7 @@
       <c r="N166" s="5"/>
       <c r="O166" s="2"/>
     </row>
-    <row r="167" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A167" s="2"/>
       <c r="B167" s="5"/>
       <c r="C167" s="2"/>
@@ -5933,7 +5935,7 @@
       <c r="N167" s="5"/>
       <c r="O167" s="2"/>
     </row>
-    <row r="168" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A168" s="2"/>
       <c r="B168" s="5"/>
       <c r="C168" s="2"/>
@@ -5949,7 +5951,7 @@
       <c r="N168" s="5"/>
       <c r="O168" s="2"/>
     </row>
-    <row r="169" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A169" s="2"/>
       <c r="B169" s="5"/>
       <c r="C169" s="2"/>
@@ -5965,7 +5967,7 @@
       <c r="N169" s="5"/>
       <c r="O169" s="2"/>
     </row>
-    <row r="170" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A170" s="2"/>
       <c r="B170" s="5"/>
       <c r="C170" s="2"/>
@@ -5981,7 +5983,7 @@
       <c r="N170" s="5"/>
       <c r="O170" s="2"/>
     </row>
-    <row r="171" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A171" s="2"/>
       <c r="B171" s="5"/>
       <c r="C171" s="2"/>
@@ -5997,7 +5999,7 @@
       <c r="N171" s="5"/>
       <c r="O171" s="2"/>
     </row>
-    <row r="172" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A172" s="2"/>
       <c r="B172" s="5"/>
       <c r="C172" s="2"/>
@@ -6013,7 +6015,7 @@
       <c r="N172" s="5"/>
       <c r="O172" s="2"/>
     </row>
-    <row r="173" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A173" s="2"/>
       <c r="B173" s="5"/>
       <c r="C173" s="2"/>
@@ -6029,7 +6031,7 @@
       <c r="N173" s="5"/>
       <c r="O173" s="2"/>
     </row>
-    <row r="174" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A174" s="2"/>
       <c r="B174" s="5"/>
       <c r="C174" s="2"/>
@@ -6045,7 +6047,7 @@
       <c r="N174" s="5"/>
       <c r="O174" s="2"/>
     </row>
-    <row r="175" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A175" s="2"/>
       <c r="B175" s="5"/>
       <c r="C175" s="2"/>
@@ -6061,7 +6063,7 @@
       <c r="N175" s="5"/>
       <c r="O175" s="2"/>
     </row>
-    <row r="176" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A176" s="2"/>
       <c r="B176" s="5"/>
       <c r="C176" s="2"/>
@@ -6077,7 +6079,7 @@
       <c r="N176" s="5"/>
       <c r="O176" s="2"/>
     </row>
-    <row r="177" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A177" s="2"/>
       <c r="B177" s="5"/>
       <c r="C177" s="2"/>
@@ -6093,7 +6095,7 @@
       <c r="N177" s="5"/>
       <c r="O177" s="2"/>
     </row>
-    <row r="178" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A178" s="2"/>
       <c r="B178" s="5"/>
       <c r="C178" s="2"/>
@@ -6109,7 +6111,7 @@
       <c r="N178" s="5"/>
       <c r="O178" s="2"/>
     </row>
-    <row r="179" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A179" s="2"/>
       <c r="B179" s="5"/>
       <c r="C179" s="2"/>
@@ -6125,7 +6127,7 @@
       <c r="N179" s="5"/>
       <c r="O179" s="2"/>
     </row>
-    <row r="180" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A180" s="2"/>
       <c r="B180" s="5"/>
       <c r="C180" s="2"/>
@@ -6141,7 +6143,7 @@
       <c r="N180" s="5"/>
       <c r="O180" s="2"/>
     </row>
-    <row r="181" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A181" s="2"/>
       <c r="B181" s="5"/>
       <c r="C181" s="2"/>
@@ -6157,7 +6159,7 @@
       <c r="N181" s="5"/>
       <c r="O181" s="2"/>
     </row>
-    <row r="182" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A182" s="2"/>
       <c r="B182" s="5"/>
       <c r="C182" s="2"/>
@@ -6173,7 +6175,7 @@
       <c r="N182" s="5"/>
       <c r="O182" s="2"/>
     </row>
-    <row r="183" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A183" s="2"/>
       <c r="B183" s="5"/>
       <c r="C183" s="2"/>
@@ -6189,7 +6191,7 @@
       <c r="N183" s="5"/>
       <c r="O183" s="2"/>
     </row>
-    <row r="184" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A184" s="2"/>
       <c r="B184" s="5"/>
       <c r="C184" s="2"/>
@@ -6205,7 +6207,7 @@
       <c r="N184" s="5"/>
       <c r="O184" s="2"/>
     </row>
-    <row r="185" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A185" s="2"/>
       <c r="B185" s="5"/>
       <c r="C185" s="2"/>
@@ -6221,7 +6223,7 @@
       <c r="N185" s="5"/>
       <c r="O185" s="2"/>
     </row>
-    <row r="186" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A186" s="2"/>
       <c r="B186" s="5"/>
       <c r="C186" s="2"/>
@@ -6237,7 +6239,7 @@
       <c r="N186" s="5"/>
       <c r="O186" s="2"/>
     </row>
-    <row r="187" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A187" s="2"/>
       <c r="B187" s="5"/>
       <c r="C187" s="2"/>
@@ -6253,7 +6255,7 @@
       <c r="N187" s="5"/>
       <c r="O187" s="2"/>
     </row>
-    <row r="188" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A188" s="2"/>
       <c r="B188" s="5"/>
       <c r="C188" s="2"/>
@@ -6269,7 +6271,7 @@
       <c r="N188" s="5"/>
       <c r="O188" s="2"/>
     </row>
-    <row r="189" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A189" s="2"/>
       <c r="B189" s="5"/>
       <c r="C189" s="2"/>
@@ -6285,7 +6287,7 @@
       <c r="N189" s="5"/>
       <c r="O189" s="2"/>
     </row>
-    <row r="190" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A190" s="2"/>
       <c r="B190" s="5"/>
       <c r="C190" s="2"/>
@@ -6301,7 +6303,7 @@
       <c r="N190" s="5"/>
       <c r="O190" s="2"/>
     </row>
-    <row r="191" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A191" s="2"/>
       <c r="B191" s="5"/>
       <c r="C191" s="2"/>
@@ -6317,7 +6319,7 @@
       <c r="N191" s="5"/>
       <c r="O191" s="2"/>
     </row>
-    <row r="192" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A192" s="2"/>
       <c r="B192" s="5"/>
       <c r="C192" s="2"/>
@@ -6333,7 +6335,7 @@
       <c r="N192" s="5"/>
       <c r="O192" s="2"/>
     </row>
-    <row r="193" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A193" s="2"/>
       <c r="B193" s="5"/>
       <c r="C193" s="2"/>
@@ -6349,7 +6351,7 @@
       <c r="N193" s="5"/>
       <c r="O193" s="2"/>
     </row>
-    <row r="194" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A194" s="2"/>
       <c r="B194" s="5"/>
       <c r="C194" s="2"/>
@@ -6365,7 +6367,7 @@
       <c r="N194" s="5"/>
       <c r="O194" s="2"/>
     </row>
-    <row r="195" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A195" s="2"/>
       <c r="B195" s="5"/>
       <c r="C195" s="2"/>
@@ -6381,7 +6383,7 @@
       <c r="N195" s="5"/>
       <c r="O195" s="2"/>
     </row>
-    <row r="196" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A196" s="2"/>
       <c r="B196" s="5"/>
       <c r="C196" s="2"/>
@@ -6397,7 +6399,7 @@
       <c r="N196" s="5"/>
       <c r="O196" s="2"/>
     </row>
-    <row r="197" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A197" s="2"/>
       <c r="B197" s="5"/>
       <c r="C197" s="2"/>
@@ -6413,7 +6415,7 @@
       <c r="N197" s="5"/>
       <c r="O197" s="2"/>
     </row>
-    <row r="198" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A198" s="2"/>
       <c r="B198" s="5"/>
       <c r="C198" s="2"/>
@@ -6429,7 +6431,7 @@
       <c r="N198" s="5"/>
       <c r="O198" s="2"/>
     </row>
-    <row r="199" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A199" s="2"/>
       <c r="B199" s="5"/>
       <c r="C199" s="2"/>
@@ -6445,7 +6447,7 @@
       <c r="N199" s="5"/>
       <c r="O199" s="2"/>
     </row>
-    <row r="200" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A200" s="2"/>
       <c r="B200" s="5"/>
       <c r="C200" s="2"/>
@@ -6461,7 +6463,7 @@
       <c r="N200" s="5"/>
       <c r="O200" s="2"/>
     </row>
-    <row r="201" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A201" s="2"/>
       <c r="B201" s="5"/>
       <c r="C201" s="2"/>
@@ -6477,7 +6479,7 @@
       <c r="N201" s="5"/>
       <c r="O201" s="2"/>
     </row>
-    <row r="202" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A202" s="2"/>
       <c r="B202" s="5"/>
       <c r="C202" s="2"/>
@@ -6493,7 +6495,7 @@
       <c r="N202" s="5"/>
       <c r="O202" s="2"/>
     </row>
-    <row r="203" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A203" s="2"/>
       <c r="B203" s="5"/>
       <c r="C203" s="2"/>
@@ -6509,7 +6511,7 @@
       <c r="N203" s="5"/>
       <c r="O203" s="2"/>
     </row>
-    <row r="204" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A204" s="2"/>
       <c r="B204" s="5"/>
       <c r="C204" s="2"/>
@@ -6525,7 +6527,7 @@
       <c r="N204" s="5"/>
       <c r="O204" s="2"/>
     </row>
-    <row r="205" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A205" s="2"/>
       <c r="B205" s="5"/>
       <c r="C205" s="2"/>
@@ -6541,7 +6543,7 @@
       <c r="N205" s="5"/>
       <c r="O205" s="2"/>
     </row>
-    <row r="206" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A206" s="2"/>
       <c r="B206" s="5"/>
       <c r="C206" s="2"/>
@@ -6557,7 +6559,7 @@
       <c r="N206" s="5"/>
       <c r="O206" s="2"/>
     </row>
-    <row r="207" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A207" s="2"/>
       <c r="B207" s="5"/>
       <c r="C207" s="2"/>
@@ -6573,7 +6575,7 @@
       <c r="N207" s="5"/>
       <c r="O207" s="2"/>
     </row>
-    <row r="208" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A208" s="2"/>
       <c r="B208" s="5"/>
       <c r="C208" s="2"/>
@@ -6589,7 +6591,7 @@
       <c r="N208" s="5"/>
       <c r="O208" s="2"/>
     </row>
-    <row r="209" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A209" s="2"/>
       <c r="B209" s="5"/>
       <c r="C209" s="2"/>
@@ -6605,7 +6607,7 @@
       <c r="N209" s="5"/>
       <c r="O209" s="2"/>
     </row>
-    <row r="210" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A210" s="2"/>
       <c r="B210" s="5"/>
       <c r="C210" s="2"/>
@@ -6621,7 +6623,7 @@
       <c r="N210" s="5"/>
       <c r="O210" s="2"/>
     </row>
-    <row r="211" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A211" s="2"/>
       <c r="B211" s="5"/>
       <c r="C211" s="2"/>
@@ -6637,7 +6639,7 @@
       <c r="N211" s="5"/>
       <c r="O211" s="2"/>
     </row>
-    <row r="212" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A212" s="2"/>
       <c r="B212" s="5"/>
       <c r="C212" s="2"/>
@@ -6653,7 +6655,7 @@
       <c r="N212" s="5"/>
       <c r="O212" s="2"/>
     </row>
-    <row r="213" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A213" s="2"/>
       <c r="B213" s="5"/>
       <c r="C213" s="2"/>
@@ -6669,7 +6671,7 @@
       <c r="N213" s="5"/>
       <c r="O213" s="2"/>
     </row>
-    <row r="214" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A214" s="2"/>
       <c r="B214" s="5"/>
       <c r="C214" s="2"/>
@@ -6685,7 +6687,7 @@
       <c r="N214" s="5"/>
       <c r="O214" s="2"/>
     </row>
-    <row r="215" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A215" s="2"/>
       <c r="B215" s="5"/>
       <c r="C215" s="2"/>
@@ -6701,7 +6703,7 @@
       <c r="N215" s="5"/>
       <c r="O215" s="2"/>
     </row>
-    <row r="216" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A216" s="2"/>
       <c r="B216" s="5"/>
       <c r="C216" s="2"/>
@@ -6717,7 +6719,7 @@
       <c r="N216" s="5"/>
       <c r="O216" s="2"/>
     </row>
-    <row r="217" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A217" s="2"/>
       <c r="B217" s="5"/>
       <c r="C217" s="2"/>
@@ -6733,7 +6735,7 @@
       <c r="N217" s="5"/>
       <c r="O217" s="2"/>
     </row>
-    <row r="218" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A218" s="2"/>
       <c r="B218" s="5"/>
       <c r="C218" s="2"/>
@@ -6749,7 +6751,7 @@
       <c r="N218" s="5"/>
       <c r="O218" s="2"/>
     </row>
-    <row r="219" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A219" s="2"/>
       <c r="B219" s="5"/>
       <c r="C219" s="2"/>
@@ -6765,7 +6767,7 @@
       <c r="N219" s="5"/>
       <c r="O219" s="2"/>
     </row>
-    <row r="220" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A220" s="2"/>
       <c r="B220" s="5"/>
       <c r="C220" s="2"/>
@@ -6781,7 +6783,7 @@
       <c r="N220" s="5"/>
       <c r="O220" s="2"/>
     </row>
-    <row r="221" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A221" s="2"/>
       <c r="B221" s="5"/>
       <c r="C221" s="2"/>
@@ -6797,7 +6799,7 @@
       <c r="N221" s="5"/>
       <c r="O221" s="2"/>
     </row>
-    <row r="222" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A222" s="2"/>
       <c r="B222" s="5"/>
       <c r="C222" s="2"/>
@@ -6813,7 +6815,7 @@
       <c r="N222" s="5"/>
       <c r="O222" s="2"/>
     </row>
-    <row r="223" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A223" s="2"/>
       <c r="B223" s="5"/>
       <c r="C223" s="2"/>
@@ -6829,7 +6831,7 @@
       <c r="N223" s="5"/>
       <c r="O223" s="2"/>
     </row>
-    <row r="224" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A224" s="2"/>
       <c r="B224" s="5"/>
       <c r="C224" s="2"/>
@@ -6845,7 +6847,7 @@
       <c r="N224" s="5"/>
       <c r="O224" s="2"/>
     </row>
-    <row r="225" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A225" s="2"/>
       <c r="B225" s="5"/>
       <c r="C225" s="2"/>
@@ -6861,7 +6863,7 @@
       <c r="N225" s="5"/>
       <c r="O225" s="2"/>
     </row>
-    <row r="226" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A226" s="2"/>
       <c r="B226" s="5"/>
       <c r="C226" s="2"/>
@@ -6877,7 +6879,7 @@
       <c r="N226" s="5"/>
       <c r="O226" s="2"/>
     </row>
-    <row r="227" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A227" s="2"/>
       <c r="B227" s="5"/>
       <c r="C227" s="2"/>
@@ -6893,7 +6895,7 @@
       <c r="N227" s="5"/>
       <c r="O227" s="2"/>
     </row>
-    <row r="228" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A228" s="2"/>
       <c r="B228" s="5"/>
       <c r="C228" s="2"/>
@@ -6909,7 +6911,7 @@
       <c r="N228" s="5"/>
       <c r="O228" s="2"/>
     </row>
-    <row r="229" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A229" s="2"/>
       <c r="B229" s="5"/>
       <c r="C229" s="2"/>
@@ -6925,7 +6927,7 @@
       <c r="N229" s="5"/>
       <c r="O229" s="2"/>
     </row>
-    <row r="230" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A230" s="2"/>
       <c r="B230" s="5"/>
       <c r="C230" s="2"/>
@@ -6941,7 +6943,7 @@
       <c r="N230" s="5"/>
       <c r="O230" s="2"/>
     </row>
-    <row r="231" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A231" s="2"/>
       <c r="B231" s="5"/>
       <c r="C231" s="2"/>
@@ -6957,7 +6959,7 @@
       <c r="N231" s="5"/>
       <c r="O231" s="2"/>
     </row>
-    <row r="232" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A232" s="2"/>
       <c r="B232" s="5"/>
       <c r="C232" s="2"/>
@@ -6973,7 +6975,7 @@
       <c r="N232" s="5"/>
       <c r="O232" s="2"/>
     </row>
-    <row r="233" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A233" s="2"/>
       <c r="B233" s="5"/>
       <c r="C233" s="2"/>
@@ -6989,7 +6991,7 @@
       <c r="N233" s="5"/>
       <c r="O233" s="2"/>
     </row>
-    <row r="234" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A234" s="2"/>
       <c r="B234" s="5"/>
       <c r="C234" s="2"/>
@@ -7005,7 +7007,7 @@
       <c r="N234" s="5"/>
       <c r="O234" s="2"/>
     </row>
-    <row r="235" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A235" s="2"/>
       <c r="B235" s="5"/>
       <c r="C235" s="2"/>
@@ -7021,7 +7023,7 @@
       <c r="N235" s="5"/>
       <c r="O235" s="2"/>
     </row>
-    <row r="236" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A236" s="2"/>
       <c r="B236" s="5"/>
       <c r="C236" s="2"/>
@@ -7037,7 +7039,7 @@
       <c r="N236" s="5"/>
       <c r="O236" s="2"/>
     </row>
-    <row r="237" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A237" s="2"/>
       <c r="B237" s="5"/>
       <c r="C237" s="2"/>
@@ -7053,7 +7055,7 @@
       <c r="N237" s="5"/>
       <c r="O237" s="2"/>
     </row>
-    <row r="238" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A238" s="2"/>
       <c r="B238" s="5"/>
       <c r="C238" s="2"/>
@@ -7069,7 +7071,7 @@
       <c r="N238" s="5"/>
       <c r="O238" s="2"/>
     </row>
-    <row r="239" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A239" s="2"/>
       <c r="B239" s="5"/>
       <c r="C239" s="2"/>
@@ -7085,7 +7087,7 @@
       <c r="N239" s="5"/>
       <c r="O239" s="2"/>
     </row>
-    <row r="240" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A240" s="2"/>
       <c r="B240" s="5"/>
       <c r="C240" s="2"/>
@@ -7101,7 +7103,7 @@
       <c r="N240" s="5"/>
       <c r="O240" s="2"/>
     </row>
-    <row r="241" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A241" s="2"/>
       <c r="B241" s="5"/>
       <c r="C241" s="2"/>
@@ -7117,7 +7119,7 @@
       <c r="N241" s="5"/>
       <c r="O241" s="2"/>
     </row>
-    <row r="242" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A242" s="2"/>
       <c r="B242" s="5"/>
       <c r="C242" s="2"/>
@@ -7133,7 +7135,7 @@
       <c r="N242" s="5"/>
       <c r="O242" s="2"/>
     </row>
-    <row r="243" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A243" s="2"/>
       <c r="B243" s="5"/>
       <c r="C243" s="2"/>
@@ -7149,7 +7151,7 @@
       <c r="N243" s="5"/>
       <c r="O243" s="2"/>
     </row>
-    <row r="244" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A244" s="2"/>
       <c r="B244" s="5"/>
       <c r="C244" s="2"/>
@@ -7165,7 +7167,7 @@
       <c r="N244" s="5"/>
       <c r="O244" s="2"/>
     </row>
-    <row r="245" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A245" s="2"/>
       <c r="B245" s="5"/>
       <c r="C245" s="2"/>
@@ -7181,7 +7183,7 @@
       <c r="N245" s="5"/>
       <c r="O245" s="2"/>
     </row>
-    <row r="246" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A246" s="2"/>
       <c r="B246" s="5"/>
       <c r="C246" s="2"/>
@@ -7197,7 +7199,7 @@
       <c r="N246" s="5"/>
       <c r="O246" s="2"/>
     </row>
-    <row r="247" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A247" s="2"/>
       <c r="B247" s="5"/>
       <c r="C247" s="2"/>
@@ -7213,7 +7215,7 @@
       <c r="N247" s="5"/>
       <c r="O247" s="2"/>
     </row>
-    <row r="248" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A248" s="2"/>
       <c r="B248" s="5"/>
       <c r="C248" s="2"/>
@@ -7229,7 +7231,7 @@
       <c r="N248" s="5"/>
       <c r="O248" s="2"/>
     </row>
-    <row r="249" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A249" s="2"/>
       <c r="B249" s="5"/>
       <c r="C249" s="2"/>
@@ -7245,7 +7247,7 @@
       <c r="N249" s="5"/>
       <c r="O249" s="2"/>
     </row>
-    <row r="250" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A250" s="2"/>
       <c r="B250" s="5"/>
       <c r="C250" s="2"/>
@@ -7261,7 +7263,7 @@
       <c r="N250" s="5"/>
       <c r="O250" s="2"/>
     </row>
-    <row r="251" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A251" s="2"/>
       <c r="B251" s="5"/>
       <c r="C251" s="2"/>
@@ -7277,7 +7279,7 @@
       <c r="N251" s="5"/>
       <c r="O251" s="2"/>
     </row>
-    <row r="252" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A252" s="2"/>
       <c r="B252" s="5"/>
       <c r="C252" s="2"/>
@@ -7293,7 +7295,7 @@
       <c r="N252" s="5"/>
       <c r="O252" s="2"/>
     </row>
-    <row r="253" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A253" s="2"/>
       <c r="B253" s="5"/>
       <c r="C253" s="2"/>
@@ -7309,7 +7311,7 @@
       <c r="N253" s="5"/>
       <c r="O253" s="2"/>
     </row>
-    <row r="254" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A254" s="2"/>
       <c r="B254" s="5"/>
       <c r="C254" s="2"/>
@@ -7325,7 +7327,7 @@
       <c r="N254" s="5"/>
       <c r="O254" s="2"/>
     </row>
-    <row r="255" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A255" s="2"/>
       <c r="B255" s="5"/>
       <c r="C255" s="2"/>
@@ -7341,7 +7343,7 @@
       <c r="N255" s="5"/>
       <c r="O255" s="2"/>
     </row>
-    <row r="256" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A256" s="2"/>
       <c r="B256" s="5"/>
       <c r="C256" s="2"/>
@@ -7357,7 +7359,7 @@
       <c r="N256" s="5"/>
       <c r="O256" s="2"/>
     </row>
-    <row r="257" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A257" s="2"/>
       <c r="B257" s="5"/>
       <c r="C257" s="2"/>
@@ -7373,7 +7375,7 @@
       <c r="N257" s="5"/>
       <c r="O257" s="2"/>
     </row>
-    <row r="258" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A258" s="2"/>
       <c r="B258" s="5"/>
       <c r="C258" s="2"/>
@@ -7389,7 +7391,7 @@
       <c r="N258" s="5"/>
       <c r="O258" s="2"/>
     </row>
-    <row r="259" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A259" s="2"/>
       <c r="B259" s="5"/>
       <c r="C259" s="2"/>
@@ -7405,7 +7407,7 @@
       <c r="N259" s="5"/>
       <c r="O259" s="2"/>
     </row>
-    <row r="260" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A260" s="2"/>
       <c r="B260" s="5"/>
       <c r="C260" s="2"/>
@@ -7421,7 +7423,7 @@
       <c r="N260" s="5"/>
       <c r="O260" s="2"/>
     </row>
-    <row r="261" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A261" s="2"/>
       <c r="B261" s="5"/>
       <c r="C261" s="2"/>
@@ -7437,7 +7439,7 @@
       <c r="N261" s="5"/>
       <c r="O261" s="2"/>
     </row>
-    <row r="262" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A262" s="2"/>
       <c r="B262" s="5"/>
       <c r="C262" s="2"/>
@@ -7453,7 +7455,7 @@
       <c r="N262" s="5"/>
       <c r="O262" s="2"/>
     </row>
-    <row r="263" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A263" s="2"/>
       <c r="B263" s="5"/>
       <c r="C263" s="2"/>
@@ -7469,7 +7471,7 @@
       <c r="N263" s="5"/>
       <c r="O263" s="2"/>
     </row>
-    <row r="264" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A264" s="2"/>
       <c r="B264" s="5"/>
       <c r="C264" s="2"/>
@@ -7485,7 +7487,7 @@
       <c r="N264" s="5"/>
       <c r="O264" s="2"/>
     </row>
-    <row r="265" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A265" s="2"/>
       <c r="B265" s="5"/>
       <c r="C265" s="2"/>
@@ -7501,7 +7503,7 @@
       <c r="N265" s="5"/>
       <c r="O265" s="2"/>
     </row>
-    <row r="266" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A266" s="2"/>
       <c r="B266" s="5"/>
       <c r="C266" s="2"/>
@@ -7517,7 +7519,7 @@
       <c r="N266" s="5"/>
       <c r="O266" s="2"/>
     </row>
-    <row r="267" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A267" s="2"/>
       <c r="B267" s="5"/>
       <c r="C267" s="2"/>
@@ -7533,7 +7535,7 @@
       <c r="N267" s="5"/>
       <c r="O267" s="2"/>
     </row>
-    <row r="268" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A268" s="2"/>
       <c r="B268" s="5"/>
       <c r="C268" s="2"/>
@@ -7549,7 +7551,7 @@
       <c r="N268" s="5"/>
       <c r="O268" s="2"/>
     </row>
-    <row r="269" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A269" s="2"/>
       <c r="B269" s="5"/>
       <c r="C269" s="2"/>
@@ -7565,7 +7567,7 @@
       <c r="N269" s="5"/>
       <c r="O269" s="2"/>
     </row>
-    <row r="270" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A270" s="2"/>
       <c r="B270" s="5"/>
       <c r="C270" s="2"/>
@@ -7581,7 +7583,7 @@
       <c r="N270" s="5"/>
       <c r="O270" s="2"/>
     </row>
-    <row r="271" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A271" s="2"/>
       <c r="B271" s="5"/>
       <c r="C271" s="2"/>
@@ -7597,7 +7599,7 @@
       <c r="N271" s="5"/>
       <c r="O271" s="2"/>
     </row>
-    <row r="272" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A272" s="2"/>
       <c r="B272" s="5"/>
       <c r="C272" s="2"/>
@@ -7613,7 +7615,7 @@
       <c r="N272" s="5"/>
       <c r="O272" s="2"/>
     </row>
-    <row r="273" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A273" s="2"/>
       <c r="B273" s="5"/>
       <c r="C273" s="2"/>
@@ -7629,7 +7631,7 @@
       <c r="N273" s="5"/>
       <c r="O273" s="2"/>
     </row>
-    <row r="274" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A274" s="2"/>
       <c r="B274" s="5"/>
       <c r="C274" s="2"/>
@@ -7645,7 +7647,7 @@
       <c r="N274" s="5"/>
       <c r="O274" s="2"/>
     </row>
-    <row r="275" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A275" s="2"/>
       <c r="B275" s="5"/>
       <c r="C275" s="2"/>
@@ -7661,7 +7663,7 @@
       <c r="N275" s="5"/>
       <c r="O275" s="2"/>
     </row>
-    <row r="276" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A276" s="2"/>
       <c r="B276" s="5"/>
       <c r="C276" s="2"/>
@@ -7677,7 +7679,7 @@
       <c r="N276" s="5"/>
       <c r="O276" s="2"/>
     </row>
-    <row r="277" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A277" s="2"/>
       <c r="B277" s="5"/>
       <c r="C277" s="2"/>
@@ -7693,7 +7695,7 @@
       <c r="N277" s="5"/>
       <c r="O277" s="2"/>
     </row>
-    <row r="278" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A278" s="2"/>
       <c r="B278" s="5"/>
       <c r="C278" s="2"/>
@@ -7709,7 +7711,7 @@
       <c r="N278" s="5"/>
       <c r="O278" s="2"/>
     </row>
-    <row r="279" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A279" s="2"/>
       <c r="B279" s="5"/>
       <c r="C279" s="2"/>
@@ -7725,7 +7727,7 @@
       <c r="N279" s="5"/>
       <c r="O279" s="2"/>
     </row>
-    <row r="280" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A280" s="2"/>
       <c r="B280" s="5"/>
       <c r="C280" s="2"/>
@@ -7741,7 +7743,7 @@
       <c r="N280" s="5"/>
       <c r="O280" s="2"/>
     </row>
-    <row r="281" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A281" s="2"/>
       <c r="B281" s="5"/>
       <c r="C281" s="2"/>
@@ -7757,7 +7759,7 @@
       <c r="N281" s="5"/>
       <c r="O281" s="2"/>
     </row>
-    <row r="282" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A282" s="2"/>
       <c r="B282" s="5"/>
       <c r="C282" s="2"/>
@@ -7773,7 +7775,7 @@
       <c r="N282" s="5"/>
       <c r="O282" s="2"/>
     </row>
-    <row r="283" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A283" s="2"/>
       <c r="B283" s="5"/>
       <c r="C283" s="2"/>
@@ -7789,7 +7791,7 @@
       <c r="N283" s="5"/>
       <c r="O283" s="2"/>
     </row>
-    <row r="284" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A284" s="2"/>
       <c r="B284" s="5"/>
       <c r="C284" s="2"/>
@@ -7805,7 +7807,7 @@
       <c r="N284" s="5"/>
       <c r="O284" s="2"/>
     </row>
-    <row r="285" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A285" s="2"/>
       <c r="B285" s="5"/>
       <c r="C285" s="2"/>
@@ -7821,7 +7823,7 @@
       <c r="N285" s="5"/>
       <c r="O285" s="2"/>
     </row>
-    <row r="286" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A286" s="2"/>
       <c r="B286" s="5"/>
       <c r="C286" s="2"/>
@@ -7837,7 +7839,7 @@
       <c r="N286" s="5"/>
       <c r="O286" s="2"/>
     </row>
-    <row r="287" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A287" s="2"/>
       <c r="B287" s="5"/>
       <c r="C287" s="2"/>
@@ -7853,7 +7855,7 @@
       <c r="N287" s="5"/>
       <c r="O287" s="2"/>
     </row>
-    <row r="288" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A288" s="2"/>
       <c r="B288" s="5"/>
       <c r="C288" s="2"/>
@@ -7869,7 +7871,7 @@
       <c r="N288" s="5"/>
       <c r="O288" s="2"/>
     </row>
-    <row r="289" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A289" s="2"/>
       <c r="B289" s="5"/>
       <c r="C289" s="2"/>
@@ -7885,7 +7887,7 @@
       <c r="N289" s="5"/>
       <c r="O289" s="2"/>
     </row>
-    <row r="290" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A290" s="2"/>
       <c r="B290" s="5"/>
       <c r="C290" s="2"/>
@@ -7901,7 +7903,7 @@
       <c r="N290" s="5"/>
       <c r="O290" s="2"/>
     </row>
-    <row r="291" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A291" s="2"/>
       <c r="B291" s="5"/>
       <c r="C291" s="2"/>
@@ -7917,7 +7919,7 @@
       <c r="N291" s="5"/>
       <c r="O291" s="2"/>
     </row>
-    <row r="292" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A292" s="2"/>
       <c r="B292" s="5"/>
       <c r="C292" s="2"/>
@@ -7933,7 +7935,7 @@
       <c r="N292" s="5"/>
       <c r="O292" s="2"/>
     </row>
-    <row r="293" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A293" s="2"/>
       <c r="B293" s="5"/>
       <c r="C293" s="2"/>
@@ -7949,7 +7951,7 @@
       <c r="N293" s="5"/>
       <c r="O293" s="2"/>
     </row>
-    <row r="294" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A294" s="2"/>
       <c r="B294" s="5"/>
       <c r="C294" s="2"/>
@@ -7965,7 +7967,7 @@
       <c r="N294" s="5"/>
       <c r="O294" s="2"/>
     </row>
-    <row r="295" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A295" s="2"/>
       <c r="B295" s="5"/>
       <c r="C295" s="2"/>
@@ -7981,7 +7983,7 @@
       <c r="N295" s="5"/>
       <c r="O295" s="2"/>
     </row>
-    <row r="296" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A296" s="2"/>
       <c r="B296" s="5"/>
       <c r="C296" s="2"/>
@@ -7997,7 +7999,7 @@
       <c r="N296" s="5"/>
       <c r="O296" s="2"/>
     </row>
-    <row r="297" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A297" s="2"/>
       <c r="B297" s="5"/>
       <c r="C297" s="2"/>
@@ -8013,7 +8015,7 @@
       <c r="N297" s="5"/>
       <c r="O297" s="2"/>
     </row>
-    <row r="298" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A298" s="2"/>
       <c r="B298" s="5"/>
       <c r="C298" s="2"/>
@@ -8029,7 +8031,7 @@
       <c r="N298" s="5"/>
       <c r="O298" s="2"/>
     </row>
-    <row r="299" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="299" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A299" s="2"/>
       <c r="B299" s="5"/>
       <c r="C299" s="2"/>
@@ -8045,7 +8047,7 @@
       <c r="N299" s="5"/>
       <c r="O299" s="2"/>
     </row>
-    <row r="300" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A300" s="2"/>
       <c r="B300" s="5"/>
       <c r="C300" s="2"/>
@@ -8061,7 +8063,7 @@
       <c r="N300" s="5"/>
       <c r="O300" s="2"/>
     </row>
-    <row r="301" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A301" s="2"/>
       <c r="B301" s="5"/>
       <c r="C301" s="2"/>
@@ -8077,7 +8079,7 @@
       <c r="N301" s="5"/>
       <c r="O301" s="2"/>
     </row>
-    <row r="302" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="302" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A302" s="2"/>
       <c r="B302" s="5"/>
       <c r="C302" s="2"/>
@@ -8093,7 +8095,7 @@
       <c r="N302" s="5"/>
       <c r="O302" s="2"/>
     </row>
-    <row r="303" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A303" s="2"/>
       <c r="B303" s="5"/>
       <c r="C303" s="2"/>
@@ -8109,7 +8111,7 @@
       <c r="N303" s="5"/>
       <c r="O303" s="2"/>
     </row>
-    <row r="304" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A304" s="2"/>
       <c r="B304" s="5"/>
       <c r="C304" s="2"/>
@@ -8125,7 +8127,7 @@
       <c r="N304" s="5"/>
       <c r="O304" s="2"/>
     </row>
-    <row r="305" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A305" s="2"/>
       <c r="B305" s="5"/>
       <c r="C305" s="2"/>
@@ -8141,7 +8143,7 @@
       <c r="N305" s="5"/>
       <c r="O305" s="2"/>
     </row>
-    <row r="306" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="306" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A306" s="2"/>
       <c r="B306" s="5"/>
       <c r="C306" s="2"/>
@@ -8157,7 +8159,7 @@
       <c r="N306" s="5"/>
       <c r="O306" s="2"/>
     </row>
-    <row r="307" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="307" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A307" s="2"/>
       <c r="B307" s="5"/>
       <c r="C307" s="2"/>
@@ -8173,7 +8175,7 @@
       <c r="N307" s="5"/>
       <c r="O307" s="2"/>
     </row>
-    <row r="308" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="308" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A308" s="2"/>
       <c r="B308" s="5"/>
       <c r="C308" s="2"/>
@@ -8189,7 +8191,7 @@
       <c r="N308" s="5"/>
       <c r="O308" s="2"/>
     </row>
-    <row r="309" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="309" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A309" s="2"/>
       <c r="B309" s="5"/>
       <c r="C309" s="2"/>
@@ -8205,7 +8207,7 @@
       <c r="N309" s="5"/>
       <c r="O309" s="2"/>
     </row>
-    <row r="310" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="310" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A310" s="2"/>
       <c r="B310" s="5"/>
       <c r="C310" s="2"/>
@@ -8221,7 +8223,7 @@
       <c r="N310" s="5"/>
       <c r="O310" s="2"/>
     </row>
-    <row r="311" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="311" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A311" s="2"/>
       <c r="B311" s="5"/>
       <c r="C311" s="2"/>
@@ -8237,7 +8239,7 @@
       <c r="N311" s="5"/>
       <c r="O311" s="2"/>
     </row>
-    <row r="312" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="312" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A312" s="2"/>
       <c r="B312" s="5"/>
       <c r="C312" s="2"/>
@@ -8253,7 +8255,7 @@
       <c r="N312" s="5"/>
       <c r="O312" s="2"/>
     </row>
-    <row r="313" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="313" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A313" s="2"/>
       <c r="B313" s="5"/>
       <c r="C313" s="2"/>
@@ -8269,7 +8271,7 @@
       <c r="N313" s="5"/>
       <c r="O313" s="2"/>
     </row>
-    <row r="314" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="314" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A314" s="2"/>
       <c r="B314" s="5"/>
       <c r="C314" s="2"/>
@@ -8285,7 +8287,7 @@
       <c r="N314" s="5"/>
       <c r="O314" s="2"/>
     </row>
-    <row r="315" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="315" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A315" s="2"/>
       <c r="B315" s="5"/>
       <c r="C315" s="2"/>
@@ -8301,7 +8303,7 @@
       <c r="N315" s="5"/>
       <c r="O315" s="2"/>
     </row>
-    <row r="316" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="316" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A316" s="2"/>
       <c r="B316" s="5"/>
       <c r="C316" s="2"/>
@@ -8317,7 +8319,7 @@
       <c r="N316" s="5"/>
       <c r="O316" s="2"/>
     </row>
-    <row r="317" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="317" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A317" s="2"/>
       <c r="B317" s="5"/>
       <c r="C317" s="2"/>
@@ -8333,7 +8335,7 @@
       <c r="N317" s="5"/>
       <c r="O317" s="2"/>
     </row>
-    <row r="318" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="318" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A318" s="2"/>
       <c r="B318" s="5"/>
       <c r="C318" s="2"/>
@@ -8349,7 +8351,7 @@
       <c r="N318" s="5"/>
       <c r="O318" s="2"/>
     </row>
-    <row r="319" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="319" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A319" s="2"/>
       <c r="B319" s="5"/>
       <c r="C319" s="2"/>
@@ -8365,7 +8367,7 @@
       <c r="N319" s="5"/>
       <c r="O319" s="2"/>
     </row>
-    <row r="320" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="320" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A320" s="2"/>
       <c r="B320" s="5"/>
       <c r="C320" s="2"/>
@@ -8381,7 +8383,7 @@
       <c r="N320" s="5"/>
       <c r="O320" s="2"/>
     </row>
-    <row r="321" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="321" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A321" s="2"/>
       <c r="B321" s="5"/>
       <c r="C321" s="2"/>
@@ -8397,7 +8399,7 @@
       <c r="N321" s="5"/>
       <c r="O321" s="2"/>
     </row>
-    <row r="322" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="322" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A322" s="2"/>
       <c r="B322" s="5"/>
       <c r="C322" s="2"/>
@@ -8413,7 +8415,7 @@
       <c r="N322" s="5"/>
       <c r="O322" s="2"/>
     </row>
-    <row r="323" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="323" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A323" s="2"/>
       <c r="B323" s="5"/>
       <c r="C323" s="2"/>
@@ -8429,7 +8431,7 @@
       <c r="N323" s="5"/>
       <c r="O323" s="2"/>
     </row>
-    <row r="324" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="324" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A324" s="2"/>
       <c r="B324" s="5"/>
       <c r="C324" s="2"/>
@@ -8445,7 +8447,7 @@
       <c r="N324" s="5"/>
       <c r="O324" s="2"/>
     </row>
-    <row r="325" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="325" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A325" s="2"/>
       <c r="B325" s="5"/>
       <c r="C325" s="2"/>
@@ -8461,7 +8463,7 @@
       <c r="N325" s="5"/>
       <c r="O325" s="2"/>
     </row>
-    <row r="326" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="326" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A326" s="2"/>
       <c r="B326" s="5"/>
       <c r="C326" s="2"/>
@@ -8477,7 +8479,7 @@
       <c r="N326" s="5"/>
       <c r="O326" s="2"/>
     </row>
-    <row r="327" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="327" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A327" s="2"/>
       <c r="B327" s="5"/>
       <c r="C327" s="2"/>
@@ -8493,7 +8495,7 @@
       <c r="N327" s="5"/>
       <c r="O327" s="2"/>
     </row>
-    <row r="328" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="328" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A328" s="2"/>
       <c r="B328" s="5"/>
       <c r="C328" s="2"/>
@@ -8509,7 +8511,7 @@
       <c r="N328" s="5"/>
       <c r="O328" s="2"/>
     </row>
-    <row r="329" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="329" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A329" s="2"/>
       <c r="B329" s="5"/>
       <c r="C329" s="2"/>
@@ -8525,7 +8527,7 @@
       <c r="N329" s="5"/>
       <c r="O329" s="2"/>
     </row>
-    <row r="330" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="330" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A330" s="2"/>
       <c r="B330" s="5"/>
       <c r="C330" s="2"/>
@@ -8541,7 +8543,7 @@
       <c r="N330" s="5"/>
       <c r="O330" s="2"/>
     </row>
-    <row r="331" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="331" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A331" s="2"/>
       <c r="B331" s="5"/>
       <c r="C331" s="2"/>
@@ -8557,7 +8559,7 @@
       <c r="N331" s="5"/>
       <c r="O331" s="2"/>
     </row>
-    <row r="332" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="332" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A332" s="2"/>
       <c r="B332" s="5"/>
       <c r="C332" s="2"/>
@@ -8573,7 +8575,7 @@
       <c r="N332" s="5"/>
       <c r="O332" s="2"/>
     </row>
-    <row r="333" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="333" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A333" s="2"/>
       <c r="B333" s="5"/>
       <c r="C333" s="2"/>
@@ -8589,7 +8591,7 @@
       <c r="N333" s="5"/>
       <c r="O333" s="2"/>
     </row>
-    <row r="334" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="334" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A334" s="2"/>
       <c r="B334" s="5"/>
       <c r="C334" s="2"/>
@@ -8605,7 +8607,7 @@
       <c r="N334" s="5"/>
       <c r="O334" s="2"/>
     </row>
-    <row r="335" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="335" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A335" s="2"/>
       <c r="B335" s="5"/>
       <c r="C335" s="2"/>
@@ -8621,7 +8623,7 @@
       <c r="N335" s="5"/>
       <c r="O335" s="2"/>
     </row>
-    <row r="336" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="336" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A336" s="2"/>
       <c r="B336" s="5"/>
       <c r="C336" s="2"/>
@@ -8637,7 +8639,7 @@
       <c r="N336" s="5"/>
       <c r="O336" s="2"/>
     </row>
-    <row r="337" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="337" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A337" s="2"/>
       <c r="B337" s="5"/>
       <c r="C337" s="2"/>
@@ -8653,7 +8655,7 @@
       <c r="N337" s="5"/>
       <c r="O337" s="2"/>
     </row>
-    <row r="338" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="338" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A338" s="2"/>
       <c r="B338" s="5"/>
       <c r="C338" s="2"/>
@@ -8669,7 +8671,7 @@
       <c r="N338" s="5"/>
       <c r="O338" s="2"/>
     </row>
-    <row r="339" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="339" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A339" s="2"/>
       <c r="B339" s="5"/>
       <c r="C339" s="2"/>
@@ -8685,7 +8687,7 @@
       <c r="N339" s="5"/>
       <c r="O339" s="2"/>
     </row>
-    <row r="340" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="340" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A340" s="2"/>
       <c r="B340" s="5"/>
       <c r="C340" s="2"/>
@@ -8701,7 +8703,7 @@
       <c r="N340" s="5"/>
       <c r="O340" s="2"/>
     </row>
-    <row r="341" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="341" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A341" s="2"/>
       <c r="B341" s="5"/>
       <c r="C341" s="2"/>
@@ -8717,7 +8719,7 @@
       <c r="N341" s="5"/>
       <c r="O341" s="2"/>
     </row>
-    <row r="342" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="342" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A342" s="2"/>
       <c r="B342" s="5"/>
       <c r="C342" s="2"/>
@@ -8733,7 +8735,7 @@
       <c r="N342" s="5"/>
       <c r="O342" s="2"/>
     </row>
-    <row r="343" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="343" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A343" s="2"/>
       <c r="B343" s="5"/>
       <c r="C343" s="2"/>
@@ -8749,7 +8751,7 @@
       <c r="N343" s="5"/>
       <c r="O343" s="2"/>
     </row>
-    <row r="344" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="344" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A344" s="2"/>
       <c r="B344" s="5"/>
       <c r="C344" s="2"/>
@@ -8765,7 +8767,7 @@
       <c r="N344" s="5"/>
       <c r="O344" s="2"/>
     </row>
-    <row r="345" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="345" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A345" s="2"/>
       <c r="B345" s="5"/>
       <c r="C345" s="2"/>
@@ -8781,7 +8783,7 @@
       <c r="N345" s="5"/>
       <c r="O345" s="2"/>
     </row>
-    <row r="346" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="346" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A346" s="2"/>
       <c r="B346" s="5"/>
       <c r="C346" s="2"/>
@@ -8797,7 +8799,7 @@
       <c r="N346" s="5"/>
       <c r="O346" s="2"/>
     </row>
-    <row r="347" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="347" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A347" s="2"/>
       <c r="B347" s="5"/>
       <c r="C347" s="2"/>
@@ -8813,7 +8815,7 @@
       <c r="N347" s="5"/>
       <c r="O347" s="2"/>
     </row>
-    <row r="348" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="348" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A348" s="2"/>
       <c r="B348" s="5"/>
       <c r="C348" s="2"/>
@@ -8829,7 +8831,7 @@
       <c r="N348" s="5"/>
       <c r="O348" s="2"/>
     </row>
-    <row r="349" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="349" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A349" s="2"/>
       <c r="B349" s="5"/>
       <c r="C349" s="2"/>
@@ -8845,7 +8847,7 @@
       <c r="N349" s="5"/>
       <c r="O349" s="2"/>
     </row>
-    <row r="350" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="350" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A350" s="2"/>
       <c r="B350" s="5"/>
       <c r="C350" s="2"/>
@@ -8861,7 +8863,7 @@
       <c r="N350" s="5"/>
       <c r="O350" s="2"/>
     </row>
-    <row r="351" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="351" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A351" s="2"/>
       <c r="B351" s="5"/>
       <c r="C351" s="2"/>
@@ -8877,7 +8879,7 @@
       <c r="N351" s="5"/>
       <c r="O351" s="2"/>
     </row>
-    <row r="352" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="352" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A352" s="2"/>
       <c r="B352" s="5"/>
       <c r="C352" s="2"/>
@@ -8893,7 +8895,7 @@
       <c r="N352" s="5"/>
       <c r="O352" s="2"/>
     </row>
-    <row r="353" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="353" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A353" s="2"/>
       <c r="B353" s="5"/>
       <c r="C353" s="2"/>
@@ -8909,7 +8911,7 @@
       <c r="N353" s="5"/>
       <c r="O353" s="2"/>
     </row>
-    <row r="354" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="354" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A354" s="2"/>
       <c r="B354" s="5"/>
       <c r="C354" s="2"/>
@@ -8925,7 +8927,7 @@
       <c r="N354" s="5"/>
       <c r="O354" s="2"/>
     </row>
-    <row r="355" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="355" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A355" s="2"/>
       <c r="B355" s="5"/>
       <c r="C355" s="2"/>
@@ -8941,7 +8943,7 @@
       <c r="N355" s="5"/>
       <c r="O355" s="2"/>
     </row>
-    <row r="356" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="356" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A356" s="2"/>
       <c r="B356" s="5"/>
       <c r="C356" s="2"/>
@@ -8957,7 +8959,7 @@
       <c r="N356" s="5"/>
       <c r="O356" s="2"/>
     </row>
-    <row r="357" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="357" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A357" s="2"/>
       <c r="B357" s="5"/>
       <c r="C357" s="2"/>
@@ -8973,7 +8975,7 @@
       <c r="N357" s="5"/>
       <c r="O357" s="2"/>
     </row>
-    <row r="358" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="358" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A358" s="2"/>
       <c r="B358" s="5"/>
       <c r="C358" s="2"/>
@@ -8989,7 +8991,7 @@
       <c r="N358" s="5"/>
       <c r="O358" s="2"/>
     </row>
-    <row r="359" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="359" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A359" s="2"/>
       <c r="B359" s="5"/>
       <c r="C359" s="2"/>
@@ -9005,7 +9007,7 @@
       <c r="N359" s="5"/>
       <c r="O359" s="2"/>
     </row>
-    <row r="360" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="360" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A360" s="2"/>
       <c r="B360" s="5"/>
       <c r="C360" s="2"/>
@@ -9021,7 +9023,7 @@
       <c r="N360" s="5"/>
       <c r="O360" s="2"/>
     </row>
-    <row r="361" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="361" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A361" s="2"/>
       <c r="B361" s="5"/>
       <c r="C361" s="2"/>
@@ -9037,7 +9039,7 @@
       <c r="N361" s="5"/>
       <c r="O361" s="2"/>
     </row>
-    <row r="362" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="362" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A362" s="2"/>
       <c r="B362" s="5"/>
       <c r="C362" s="2"/>
@@ -9053,7 +9055,7 @@
       <c r="N362" s="5"/>
       <c r="O362" s="2"/>
     </row>
-    <row r="363" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="363" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A363" s="2"/>
       <c r="B363" s="5"/>
       <c r="C363" s="2"/>
@@ -9069,7 +9071,7 @@
       <c r="N363" s="5"/>
       <c r="O363" s="2"/>
     </row>
-    <row r="364" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="364" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A364" s="2"/>
       <c r="B364" s="5"/>
       <c r="C364" s="2"/>
@@ -9085,7 +9087,7 @@
       <c r="N364" s="5"/>
       <c r="O364" s="2"/>
     </row>
-    <row r="365" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="365" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A365" s="2"/>
       <c r="B365" s="5"/>
       <c r="C365" s="2"/>
@@ -9101,7 +9103,7 @@
       <c r="N365" s="5"/>
       <c r="O365" s="2"/>
     </row>
-    <row r="366" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="366" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A366" s="2"/>
       <c r="B366" s="5"/>
       <c r="C366" s="2"/>
@@ -9117,7 +9119,7 @@
       <c r="N366" s="5"/>
       <c r="O366" s="2"/>
     </row>
-    <row r="367" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="367" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A367" s="2"/>
       <c r="B367" s="5"/>
       <c r="C367" s="2"/>
@@ -9133,7 +9135,7 @@
       <c r="N367" s="5"/>
       <c r="O367" s="2"/>
     </row>
-    <row r="368" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="368" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A368" s="2"/>
       <c r="B368" s="5"/>
       <c r="C368" s="2"/>
@@ -9149,7 +9151,7 @@
       <c r="N368" s="5"/>
       <c r="O368" s="2"/>
     </row>
-    <row r="369" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="369" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A369" s="2"/>
       <c r="B369" s="5"/>
       <c r="C369" s="2"/>
@@ -9165,7 +9167,7 @@
       <c r="N369" s="5"/>
       <c r="O369" s="2"/>
     </row>
-    <row r="370" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="370" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A370" s="2"/>
       <c r="B370" s="5"/>
       <c r="C370" s="2"/>
@@ -9181,7 +9183,7 @@
       <c r="N370" s="5"/>
       <c r="O370" s="2"/>
     </row>
-    <row r="371" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="371" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A371" s="2"/>
       <c r="B371" s="5"/>
       <c r="C371" s="2"/>
@@ -9197,7 +9199,7 @@
       <c r="N371" s="5"/>
       <c r="O371" s="2"/>
     </row>
-    <row r="372" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="372" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A372" s="2"/>
       <c r="B372" s="5"/>
       <c r="C372" s="2"/>
@@ -9213,7 +9215,7 @@
       <c r="N372" s="5"/>
       <c r="O372" s="2"/>
     </row>
-    <row r="373" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="373" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A373" s="2"/>
       <c r="B373" s="5"/>
       <c r="C373" s="2"/>
@@ -9229,7 +9231,7 @@
       <c r="N373" s="5"/>
       <c r="O373" s="2"/>
     </row>
-    <row r="374" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="374" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A374" s="2"/>
       <c r="B374" s="5"/>
       <c r="C374" s="2"/>
@@ -9245,7 +9247,7 @@
       <c r="N374" s="5"/>
       <c r="O374" s="2"/>
     </row>
-    <row r="375" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="375" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A375" s="2"/>
       <c r="B375" s="5"/>
       <c r="C375" s="2"/>
@@ -9261,7 +9263,7 @@
       <c r="N375" s="5"/>
       <c r="O375" s="2"/>
     </row>
-    <row r="376" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="376" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A376" s="2"/>
       <c r="B376" s="5"/>
       <c r="C376" s="2"/>
@@ -9277,7 +9279,7 @@
       <c r="N376" s="5"/>
       <c r="O376" s="2"/>
     </row>
-    <row r="377" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="377" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A377" s="2"/>
       <c r="B377" s="5"/>
       <c r="C377" s="2"/>
@@ -9293,7 +9295,7 @@
       <c r="N377" s="5"/>
       <c r="O377" s="2"/>
     </row>
-    <row r="378" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="378" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A378" s="2"/>
       <c r="B378" s="5"/>
       <c r="C378" s="2"/>
@@ -9309,7 +9311,7 @@
       <c r="N378" s="5"/>
       <c r="O378" s="2"/>
     </row>
-    <row r="379" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="379" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A379" s="2"/>
       <c r="B379" s="5"/>
       <c r="C379" s="2"/>
@@ -9325,7 +9327,7 @@
       <c r="N379" s="5"/>
       <c r="O379" s="2"/>
     </row>
-    <row r="380" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="380" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A380" s="2"/>
       <c r="B380" s="5"/>
       <c r="C380" s="2"/>
@@ -9341,7 +9343,7 @@
       <c r="N380" s="5"/>
       <c r="O380" s="2"/>
     </row>
-    <row r="381" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="381" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A381" s="2"/>
       <c r="B381" s="5"/>
       <c r="C381" s="2"/>
@@ -9357,7 +9359,7 @@
       <c r="N381" s="5"/>
       <c r="O381" s="2"/>
     </row>
-    <row r="382" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="382" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A382" s="2"/>
       <c r="B382" s="5"/>
       <c r="C382" s="2"/>
@@ -9373,7 +9375,7 @@
       <c r="N382" s="5"/>
       <c r="O382" s="2"/>
     </row>
-    <row r="383" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="383" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A383" s="2"/>
       <c r="B383" s="5"/>
       <c r="C383" s="2"/>
@@ -9389,7 +9391,7 @@
       <c r="N383" s="5"/>
       <c r="O383" s="2"/>
     </row>
-    <row r="384" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="384" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A384" s="2"/>
       <c r="B384" s="5"/>
       <c r="C384" s="2"/>
@@ -9405,7 +9407,7 @@
       <c r="N384" s="5"/>
       <c r="O384" s="2"/>
     </row>
-    <row r="385" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="385" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A385" s="2"/>
       <c r="B385" s="5"/>
       <c r="C385" s="2"/>
@@ -9421,7 +9423,7 @@
       <c r="N385" s="5"/>
       <c r="O385" s="2"/>
     </row>
-    <row r="386" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="386" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A386" s="2"/>
       <c r="B386" s="5"/>
       <c r="C386" s="2"/>
@@ -9437,7 +9439,7 @@
       <c r="N386" s="5"/>
       <c r="O386" s="2"/>
     </row>
-    <row r="387" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="387" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A387" s="2"/>
       <c r="B387" s="5"/>
       <c r="C387" s="2"/>
@@ -9453,7 +9455,7 @@
       <c r="N387" s="5"/>
       <c r="O387" s="2"/>
     </row>
-    <row r="388" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="388" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A388" s="2"/>
       <c r="B388" s="5"/>
       <c r="C388" s="2"/>
@@ -9469,7 +9471,7 @@
       <c r="N388" s="5"/>
       <c r="O388" s="2"/>
     </row>
-    <row r="389" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="389" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A389" s="2"/>
       <c r="B389" s="5"/>
       <c r="C389" s="2"/>
@@ -9485,7 +9487,7 @@
       <c r="N389" s="5"/>
       <c r="O389" s="2"/>
     </row>
-    <row r="390" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="390" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A390" s="2"/>
       <c r="B390" s="5"/>
       <c r="C390" s="2"/>
@@ -9501,7 +9503,7 @@
       <c r="N390" s="5"/>
       <c r="O390" s="2"/>
     </row>
-    <row r="391" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="391" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A391" s="2"/>
       <c r="B391" s="5"/>
       <c r="C391" s="2"/>
@@ -9517,7 +9519,7 @@
       <c r="N391" s="5"/>
       <c r="O391" s="2"/>
     </row>
-    <row r="392" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="392" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A392" s="2"/>
       <c r="B392" s="5"/>
       <c r="C392" s="2"/>
@@ -9533,7 +9535,7 @@
       <c r="N392" s="5"/>
       <c r="O392" s="2"/>
     </row>
-    <row r="393" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="393" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A393" s="2"/>
       <c r="B393" s="5"/>
       <c r="C393" s="2"/>
@@ -9549,7 +9551,7 @@
       <c r="N393" s="5"/>
       <c r="O393" s="2"/>
     </row>
-    <row r="394" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="394" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A394" s="2"/>
       <c r="B394" s="5"/>
       <c r="C394" s="2"/>
@@ -9565,7 +9567,7 @@
       <c r="N394" s="5"/>
       <c r="O394" s="2"/>
     </row>
-    <row r="395" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="395" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A395" s="2"/>
       <c r="B395" s="5"/>
       <c r="C395" s="2"/>
@@ -9581,7 +9583,7 @@
       <c r="N395" s="5"/>
       <c r="O395" s="2"/>
     </row>
-    <row r="396" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="396" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A396" s="2"/>
       <c r="B396" s="5"/>
       <c r="C396" s="2"/>
@@ -9597,7 +9599,7 @@
       <c r="N396" s="5"/>
       <c r="O396" s="2"/>
     </row>
-    <row r="397" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="397" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A397" s="2"/>
       <c r="B397" s="5"/>
       <c r="C397" s="2"/>
@@ -9613,7 +9615,7 @@
       <c r="N397" s="5"/>
       <c r="O397" s="2"/>
     </row>
-    <row r="398" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="398" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A398" s="2"/>
       <c r="B398" s="5"/>
       <c r="C398" s="2"/>
@@ -9629,7 +9631,7 @@
       <c r="N398" s="5"/>
       <c r="O398" s="2"/>
     </row>
-    <row r="399" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="399" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A399" s="2"/>
       <c r="B399" s="5"/>
       <c r="C399" s="2"/>
@@ -9645,7 +9647,7 @@
       <c r="N399" s="5"/>
       <c r="O399" s="2"/>
     </row>
-    <row r="400" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="400" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A400" s="2"/>
       <c r="B400" s="5"/>
       <c r="C400" s="2"/>
@@ -9661,7 +9663,7 @@
       <c r="N400" s="5"/>
       <c r="O400" s="2"/>
     </row>
-    <row r="401" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="401" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A401" s="2"/>
       <c r="B401" s="5"/>
       <c r="C401" s="2"/>
@@ -9677,7 +9679,7 @@
       <c r="N401" s="5"/>
       <c r="O401" s="2"/>
     </row>
-    <row r="402" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="402" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A402" s="2"/>
       <c r="B402" s="5"/>
       <c r="C402" s="2"/>
@@ -9693,7 +9695,7 @@
       <c r="N402" s="5"/>
       <c r="O402" s="2"/>
     </row>
-    <row r="403" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="403" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A403" s="2"/>
       <c r="B403" s="5"/>
       <c r="C403" s="2"/>
@@ -9709,7 +9711,7 @@
       <c r="N403" s="5"/>
       <c r="O403" s="2"/>
     </row>
-    <row r="404" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="404" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A404" s="2"/>
       <c r="B404" s="5"/>
       <c r="C404" s="2"/>
@@ -9725,7 +9727,7 @@
       <c r="N404" s="5"/>
       <c r="O404" s="2"/>
     </row>
-    <row r="405" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="405" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A405" s="2"/>
       <c r="B405" s="5"/>
       <c r="C405" s="2"/>
@@ -9741,7 +9743,7 @@
       <c r="N405" s="5"/>
       <c r="O405" s="2"/>
     </row>
-    <row r="406" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="406" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A406" s="2"/>
       <c r="B406" s="5"/>
       <c r="C406" s="2"/>
@@ -9758,7 +9760,7 @@
       <c r="O406" s="2"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q81"/>
+  <autoFilter ref="A1:Q81" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
   <legacyDrawing r:id="rId2"/>

</xml_diff>